<commit_message>
Rebalance program schedule and align calendar with UPC holidays
- Align non-teaching dates with official UPC-FIB academic calendar
  (La Immaculada, Christmas break, UPC 9 Feb holiday)
- Rebalance M1/M5/M6 session counts: move Go from M1 into M6 right
  before building operators (just-in-time learning), split
  Observability into 3 sessions (metrics/logs/traces+correlation),
  keeping the program at 30 sessions / 90h / 12 ECTS overall
- Restructure session on application bundles (Kustomize -> Helm ->
  combined -> operator teaser) with a detailed 180-minute session
  script
- Regenerate calendario.md, .xlsx and .docx from generate_docs.py
- Add calendario-upc.pdf (official UPC calendar reference) and
  AGENT_NOTES.md (continuity notes for pending content changes)
- Add unrelated infra/codex-remote-ec2 Terraform scaffold
</commit_message>
<xml_diff>
--- a/Calendario_Postgrado_Kubernetes.xlsx
+++ b/Calendario_Postgrado_Kubernetes.xlsx
@@ -698,7 +698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -819,7 +819,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Programación asistida por IA: Bash y automatización de sistema</t>
+          <t>Bash y Python para DevOps, asistidos por IA</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
@@ -854,12 +854,12 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Python para DevOps: SDKs cloud, CLIs y testing</t>
+          <t>Redes, DNS y CDN con Cloudflare</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -894,12 +894,12 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Go para infraestructura: client-go, controllers y tooling</t>
+          <t>Control de versiones avanzado con Git</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Redes, DNS y CDN con Cloudflare</t>
+          <t>Cloud Computing: AWS, Azure y GCP</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Control de versiones avanzado con Git</t>
+          <t>Infraestructura como Código con Terraform</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
@@ -1014,12 +1014,12 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
+          <t>Contenedores y ecosistema OCI: imágenes, runtimes y seguridad</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1054,12 +1054,12 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Infraestructura como Código con Terraform</t>
+          <t>Kubernetes: arquitectura, control plane y clusters locales (kind)</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Contenedores y ecosistema OCI: imágenes, runtimes y seguridad</t>
+          <t>Building Blocks: workloads, configuración y scheduling</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Kubernetes: arquitectura, control plane y clusters locales (kind)</t>
+          <t>Almacenamiento y networking en Kubernetes</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Building Blocks: workloads, configuración y scheduling</t>
+          <t>Autenticación, RBAC y clúster componente a componente</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1214,12 +1214,12 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Almacenamiento y networking en Kubernetes</t>
+          <t>Kubernetes gestionado: EKS, GKE y AKS</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
@@ -1254,12 +1254,12 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Autenticación, RBAC y clúster componente a componente</t>
+          <t>Otros entornos y aprovisionamiento IaC multi-cloud</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>12/01/2027</t>
+          <t>22/12/2026</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Kubernetes gestionado: EKS, GKE y AKS</t>
+          <t>Application bundles: Kustomize, Helm y su ecosistema</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>14/01/2027</t>
+          <t>07/01/2027</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Otros entornos y aprovisionamiento IaC multi-cloud</t>
+          <t>Infraestructura declarativa: ExternalDNS, cert-manager y Crossplane</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>19/01/2027</t>
+          <t>12/01/2027</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Application bundles: Helm y Kustomize</t>
+          <t>Gestión de secretos: Vault y External Secrets Operator</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>21/01/2027</t>
+          <t>14/01/2027</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -1414,12 +1414,12 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura declarativa: ExternalDNS, cert-manager y Crossplane</t>
+          <t>Observabilidad (I): Prometheus, PromQL y Alertmanager</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>26/01/2027</t>
+          <t>19/01/2027</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -1454,12 +1454,12 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Gestión de secretos: Vault y External Secrets Operator</t>
+          <t>Observabilidad (II): Grafana y Loki (logs)</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>28/01/2027</t>
+          <t>21/01/2027</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Observabilidad (I): Prometheus, PromQL y Alertmanager</t>
+          <t>Observabilidad (III): OpenTelemetry, Tempo y correlación</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>02/02/2027</t>
+          <t>26/01/2027</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Observabilidad (II): Grafana stack (Loki, Tempo) y OpenTelemetry</t>
+          <t>GitOps y pipelines CI/CD: ArgoCD, Prow y Tekton</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
@@ -1559,7 +1559,7 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>04/02/2027</t>
+          <t>28/01/2027</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>GitOps y pipelines CI/CD: ArgoCD, Prow y Tekton</t>
+          <t>Networking avanzado: Traefik e Istio (service mesh)</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>09/02/2027</t>
+          <t>02/02/2027</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -1619,7 +1619,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Networking avanzado: Traefik e Istio (service mesh)</t>
+          <t>Entrega progresiva y escalado: Argo Rollouts, HPA/VPA, KEDA, Karpenter</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>11/02/2027</t>
+          <t>04/02/2027</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -1654,12 +1654,12 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M6</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Entrega progresiva y escalado: Argo Rollouts, HPA/VPA, KEDA, Karpenter</t>
+          <t>Go: de cero a controlador de Kubernetes</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -1679,12 +1679,12 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>16/02/2027</t>
+          <t>11/02/2027</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Martes</t>
+          <t>Jueves</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>18/02/2027</t>
+          <t>16/02/2027</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Jueves</t>
+          <t>Martes</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -1759,12 +1759,12 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>23/02/2027</t>
+          <t>18/02/2027</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Martes</t>
+          <t>Jueves</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
@@ -1799,12 +1799,12 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>25/02/2027</t>
+          <t>23/02/2027</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Jueves</t>
+          <t>Martes</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -1839,12 +1839,12 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>02/03/2027</t>
+          <t>25/02/2027</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Martes</t>
+          <t>Jueves</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
@@ -1879,12 +1879,12 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>04/03/2027</t>
+          <t>02/03/2027</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Jueves</t>
+          <t>Martes</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>09/03/2027</t>
+          <t>04/03/2027</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Martes</t>
+          <t>Jueves</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
@@ -1961,12 +1961,12 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>11/03/2027</t>
+          <t>09/03/2027</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Jueves</t>
+          <t>Martes</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
@@ -1999,12 +1999,12 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>16/03/2027</t>
+          <t>11/03/2027</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>Martes</t>
+          <t>Jueves</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
@@ -2037,53 +2037,91 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
+          <t>16/03/2027</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>18:00–21:00</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Reserva / recuperación</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>3h</t>
+        </is>
+      </c>
+      <c r="H34" s="9" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
           <t>18/03/2027</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C35" s="9" t="inlineStr">
         <is>
           <t>Jueves</t>
         </is>
       </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>18:00–21:00</t>
         </is>
       </c>
-      <c r="E34" s="9" t="inlineStr">
+      <c r="E35" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F35" s="5" t="inlineStr">
         <is>
           <t>Reserva / recuperación</t>
         </is>
       </c>
-      <c r="G34" s="9" t="inlineStr">
+      <c r="G35" s="9" t="inlineStr">
         <is>
           <t>3h</t>
         </is>
       </c>
-      <c r="H34" s="9" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="10" t="inlineStr">
+      <c r="H35" s="9" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B35" s="11" t="n"/>
-      <c r="C35" s="11" t="n"/>
-      <c r="D35" s="11" t="n"/>
-      <c r="E35" s="11" t="n"/>
-      <c r="F35" s="10" t="inlineStr">
+      <c r="B36" s="11" t="n"/>
+      <c r="C36" s="11" t="n"/>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="11" t="n"/>
+      <c r="F36" s="10" t="inlineStr">
         <is>
           <t>30 sesiones</t>
         </is>
       </c>
-      <c r="G35" s="11" t="n"/>
-      <c r="H35" s="10" t="inlineStr">
+      <c r="G36" s="11" t="n"/>
+      <c r="H36" s="10" t="inlineStr">
         <is>
           <t>90h</t>
         </is>
@@ -2155,12 +2193,12 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>12h</t>
+          <t>6h</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Fundamentos de DevOps y Platform Engineering · Programación para Infraestructura: Bash, Python y Go (asistida por IA)</t>
+          <t>Fundamentos de DevOps y Platform Engineering · Bash y Python para DevOps (asistida por IA)</t>
         </is>
       </c>
     </row>
@@ -2263,12 +2301,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>15h</t>
+          <t>18h</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Observabilidad · GitOps y Pipelines CI/CD · Networking Avanzado (Service Mesh) · Entrega Progresiva y Escalado</t>
+          <t>Observabilidad (I): Métricas · Observabilidad (II): Grafana y Logs · Observabilidad (III): OpenTelemetry, Tempo y Correlación · GitOps y Pipelines CI/CD · Networking Avanzado (Service Mesh) · Entrega Progresiva y Escalado</t>
         </is>
       </c>
     </row>
@@ -2290,12 +2328,12 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>15h</t>
+          <t>18h</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Construcción de Operators · Gestión de Clústeres y Serverless · Hosted Control Planes · Multi-cluster y Multi-cloud</t>
+          <t>Go: de cero a controlador de Kubernetes · Construcción de Operators · Gestión de Clústeres y Serverless · Hosted Control Planes · Multi-cluster y Multi-cloud</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C164"/>
+  <dimension ref="A1:C169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2542,7 +2580,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Programación para Infraestructura: Bash, Python y Go (asistida por IA)</t>
+          <t>Bash y Python para DevOps (asistida por IA)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -2559,12 +2597,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Programación para Infraestructura: Bash, Python y Go (asistida por IA)</t>
+          <t>Bash y Python para DevOps (asistida por IA)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Bash scripting avanzado: variables, estructuras de control, funciones, arrays y manejo de errores</t>
+          <t>Bash scripting: variables, estructuras de control, funciones, arrays y manejo de errores</t>
         </is>
       </c>
     </row>
@@ -2576,12 +2614,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Programación para Infraestructura: Bash, Python y Go (asistida por IA)</t>
+          <t>Bash y Python para DevOps (asistida por IA)</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Automatización de sistema: gestión de procesos, pipes, redirecciones, grep/sed/awk/jq/yq, cron y Makefiles</t>
+          <t>Automatización de sistema: pipes, redirecciones, grep/sed/awk/jq/yq, cron y Makefiles</t>
         </is>
       </c>
     </row>
@@ -2593,7 +2631,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Programación para Infraestructura: Bash, Python y Go (asistida por IA)</t>
+          <t>Bash y Python para DevOps (asistida por IA)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -2610,7 +2648,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Programación para Infraestructura: Bash, Python y Go (asistida por IA)</t>
+          <t>Bash y Python para DevOps (asistida por IA)</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -2627,80 +2665,80 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Programación para Infraestructura: Bash, Python y Go (asistida por IA)</t>
+          <t>Bash y Python para DevOps (asistida por IA)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Go: sintaxis, tipos, structs, interfaces, goroutines, channels y manejo de errores idiomático</t>
+          <t>Calidad de código: linting con ruff, type checking con mypy, pre-commit hooks</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>M1</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Programación para Infraestructura: Bash, Python y Go (asistida por IA)</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Go para infraestructura: desarrollo de CLIs con cobra/viper y cliente Kubernetes (client-go)</t>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Redes, DNS y CDN con Cloudflare</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Revisión de fundamentos TCP/IP, UDP, TLS 1.3/mTLS, HTTP/2 y HTTP/3 (QUIC)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>M1</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Programación para Infraestructura: Bash, Python y Go (asistida por IA)</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Patrones de desarrollo de controladores y operators en Go: reconciliation loop e informers</t>
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Redes, DNS y CDN con Cloudflare</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>DNS: resolución recursiva e iterativa, registros (A, AAAA, CNAME, TXT, SRV, NS), TTL y propagación</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>M1</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Programación para Infraestructura: Bash, Python y Go (asistida por IA)</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Testing en Go: unit tests, table-driven tests, mocks con testify e integración con CI</t>
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Redes, DNS y CDN con Cloudflare</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>DNS avanzado: DNSSEC, DNS-over-HTTPS, split-horizon DNS y service discovery basado en DNS</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>M1</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Programación para Infraestructura: Bash, Python y Go (asistida por IA)</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Herramientas de desarrollo: Makefile, direnv, pre-commit hooks y linters (golangci-lint, ruff)</t>
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Redes, DNS y CDN con Cloudflare</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>CDN: arquitectura, edge caching, routing geográfico, invalidación y cache-control headers</t>
         </is>
       </c>
     </row>
@@ -2717,7 +2755,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Revisión de fundamentos TCP/IP, UDP, TLS 1.3/mTLS, HTTP/2 y HTTP/3 (QUIC)</t>
+          <t>Cloudflare: DNS authoritative, Cloudflare Tunnel, Workers, WAF, DDoS protection y R2</t>
         </is>
       </c>
     </row>
@@ -2734,7 +2772,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>DNS: resolución recursiva e iterativa, registros (A, AAAA, CNAME, TXT, SRV, NS), TTL y propagación</t>
+          <t>Certificados TLS: PKI, cadena de confianza, ACME protocol y automatización con Let's Encrypt</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2789,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>DNS avanzado: DNSSEC, DNS-over-HTTPS, split-horizon DNS y service discovery basado en DNS</t>
+          <t>Load balancing: algoritmos, health checks, session persistence y global load balancing</t>
         </is>
       </c>
     </row>
@@ -2763,12 +2801,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Redes, DNS y CDN con Cloudflare</t>
+          <t>Control de Versiones Avanzado con Git</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>CDN: arquitectura, edge caching, routing geográfico, invalidación y cache-control headers</t>
+          <t>Arquitectura interna de Git: objects (blob, tree, commit, tag), refs, packfiles, reflog y garbage collection</t>
         </is>
       </c>
     </row>
@@ -2780,12 +2818,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Redes, DNS y CDN con Cloudflare</t>
+          <t>Control de Versiones Avanzado con Git</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Cloudflare: DNS authoritative, Cloudflare Tunnel, Workers, WAF, DDoS protection y R2</t>
+          <t>Estrategias de branching: Git Flow, GitHub Flow, trunk-based development y comparativa práctica</t>
         </is>
       </c>
     </row>
@@ -2797,12 +2835,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Redes, DNS y CDN con Cloudflare</t>
+          <t>Control de Versiones Avanzado con Git</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Certificados TLS: PKI, cadena de confianza, ACME protocol y automatización con Let's Encrypt</t>
+          <t>Rebases interactivos: squash, fixup, reword, edit y reordenación de commits</t>
         </is>
       </c>
     </row>
@@ -2814,12 +2852,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Redes, DNS y CDN con Cloudflare</t>
+          <t>Control de Versiones Avanzado con Git</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Load balancing: algoritmos, health checks, session persistence y global load balancing</t>
+          <t>Resolución de conflictos: estrategias de merge (recursive, ort), rerere, git mergetool y best practices</t>
         </is>
       </c>
     </row>
@@ -2836,7 +2874,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Arquitectura interna de Git: objects (blob, tree, commit, tag), refs, packfiles, reflog y garbage collection</t>
+          <t>Gestión de ramas: naming conventions, branch protection rules, CODEOWNERS y cleanup automático</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2891,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Estrategias de branching: Git Flow, GitHub Flow, trunk-based development y comparativa práctica</t>
+          <t>Pull Requests y code review: merge strategies (merge, squash, rebase), signed commits y draft PRs</t>
         </is>
       </c>
     </row>
@@ -2870,7 +2908,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Rebases interactivos: squash, fixup, reword, edit y reordenación de commits</t>
+          <t>Git hooks: pre-commit, commit-msg, post-merge y automatización con pre-commit framework</t>
         </is>
       </c>
     </row>
@@ -2887,7 +2925,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Resolución de conflictos: estrategias de merge (recursive, ort), rerere, git mergetool y best practices</t>
+          <t>Monorepos: estrategias, herramientas (Nx, Turborepo) y gestión de dependencias</t>
         </is>
       </c>
     </row>
@@ -2904,7 +2942,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Gestión de ramas: naming conventions, branch protection rules, CODEOWNERS y cleanup automático</t>
+          <t>Operaciones avanzadas: git bisect, git worktree, submodules, subtrees y sparse-checkout</t>
         </is>
       </c>
     </row>
@@ -2916,12 +2954,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Control de Versiones Avanzado con Git</t>
+          <t>Cloud Computing: AWS, Azure y GCP</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Pull Requests y code review: merge strategies (merge, squash, rebase), signed commits y draft PRs</t>
+          <t>AWS · IAM: users, roles, policies, OIDC federation, IRSA y AWS SSO</t>
         </is>
       </c>
     </row>
@@ -2933,12 +2971,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Control de Versiones Avanzado con Git</t>
+          <t>Cloud Computing: AWS, Azure y GCP</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Git hooks: pre-commit, commit-msg, post-merge y automatización con pre-commit framework</t>
+          <t>AWS · Computación: EC2 (instance types, AMIs, user-data), Auto Scaling Groups, Lambda</t>
         </is>
       </c>
     </row>
@@ -2950,12 +2988,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Control de Versiones Avanzado con Git</t>
+          <t>Cloud Computing: AWS, Azure y GCP</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Monorepos: estrategias, herramientas (Nx, Turborepo) y gestión de dependencias</t>
+          <t>AWS · Redes: VPC, subnets públicas/privadas, Security Groups, ALB/NLB, Route 53 y PrivateLink</t>
         </is>
       </c>
     </row>
@@ -2967,12 +3005,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Control de Versiones Avanzado con Git</t>
+          <t>Cloud Computing: AWS, Azure y GCP</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Operaciones avanzadas: git bisect, git worktree, submodules, subtrees y sparse-checkout</t>
+          <t>AWS · Almacenamiento: S3 (lifecycle, versioning), EBS, EFS y ECR</t>
         </is>
       </c>
     </row>
@@ -2989,7 +3027,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>AWS · IAM: users, roles, policies, OIDC federation, IRSA y AWS SSO</t>
+          <t>AWS · Servicios gestionados: RDS, DynamoDB, SQS, CloudWatch y Secrets Manager</t>
         </is>
       </c>
     </row>
@@ -3006,7 +3044,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>AWS · Computación: EC2 (instance types, AMIs, user-data), Auto Scaling Groups, Lambda</t>
+          <t>Azure · IAM: Entra ID, Managed Identities, RBAC y Azure Key Vault</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3061,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>AWS · Redes: VPC, subnets públicas/privadas, Security Groups, ALB/NLB, Route 53 y PrivateLink</t>
+          <t>Azure · Computación: VMs, VMSS, Azure Functions y Azure Container Apps</t>
         </is>
       </c>
     </row>
@@ -3040,7 +3078,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>AWS · Almacenamiento: S3 (lifecycle, versioning), EBS, EFS y ECR</t>
+          <t>Azure · Redes: VNet, subnets, NSG, Load Balancer, Application Gateway y Azure DNS</t>
         </is>
       </c>
     </row>
@@ -3057,7 +3095,7 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>AWS · Servicios gestionados: RDS, DynamoDB, SQS, CloudWatch y Secrets Manager</t>
+          <t>Azure · Almacenamiento: Blob Storage, Azure Files, Managed Disks y ACR</t>
         </is>
       </c>
     </row>
@@ -3074,7 +3112,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Azure · IAM: Entra ID, Managed Identities, RBAC y Azure Key Vault</t>
+          <t>Azure · Servicios gestionados: Azure SQL, Cosmos DB, Service Bus y Azure Monitor</t>
         </is>
       </c>
     </row>
@@ -3091,7 +3129,7 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Azure · Computación: VMs, VMSS, Azure Functions y Azure Container Apps</t>
+          <t>GCP · IAM: Service Accounts, Workload Identity, org policies y Cloud Audit Logs</t>
         </is>
       </c>
     </row>
@@ -3108,7 +3146,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Azure · Redes: VNet, subnets, NSG, Load Balancer, Application Gateway y Azure DNS</t>
+          <t>GCP · Computación: Compute Engine, Cloud Functions y Cloud Run</t>
         </is>
       </c>
     </row>
@@ -3125,7 +3163,7 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Azure · Almacenamiento: Blob Storage, Azure Files, Managed Disks y ACR</t>
+          <t>GCP · Redes: VPC, Firewall Rules, Cloud NAT, Cloud Load Balancing y Cloud DNS</t>
         </is>
       </c>
     </row>
@@ -3142,7 +3180,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Azure · Servicios gestionados: Azure SQL, Cosmos DB, Service Bus y Azure Monitor</t>
+          <t>GCP · Almacenamiento: Cloud Storage, Persistent Disk y Artifact Registry</t>
         </is>
       </c>
     </row>
@@ -3159,7 +3197,7 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>GCP · IAM: Service Accounts, Workload Identity, org policies y Cloud Audit Logs</t>
+          <t>GCP · Servicios gestionados: Cloud SQL, Firestore, Pub/Sub y Cloud Monitoring</t>
         </is>
       </c>
     </row>
@@ -3176,7 +3214,7 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>GCP · Computación: Compute Engine, Cloud Functions y Cloud Run</t>
+          <t>Comparativa multi-cloud: estrategias de portabilidad, vendor lock-in y abstracción de recursos</t>
         </is>
       </c>
     </row>
@@ -3188,12 +3226,12 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
+          <t>Infraestructura como Código con Terraform</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>GCP · Redes: VPC, Firewall Rules, Cloud NAT, Cloud Load Balancing y Cloud DNS</t>
+          <t>Fundamentos de IaC: filosofía declarativa vs imperativa, idempotencia y drift detection</t>
         </is>
       </c>
     </row>
@@ -3205,12 +3243,12 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
+          <t>Infraestructura como Código con Terraform</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>GCP · Almacenamiento: Cloud Storage, Persistent Disk y Artifact Registry</t>
+          <t>HCL: sintaxis, tipos de datos, expresiones, funciones y meta-argumentos (count, for_each, depends_on)</t>
         </is>
       </c>
     </row>
@@ -3222,12 +3260,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
+          <t>Infraestructura como Código con Terraform</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>GCP · Servicios gestionados: Cloud SQL, Firestore, Pub/Sub y Cloud Monitoring</t>
+          <t>Providers: configuración, autenticación y uso de los providers de AWS, Azure y GCP</t>
         </is>
       </c>
     </row>
@@ -3239,12 +3277,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
+          <t>Infraestructura como Código con Terraform</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Comparativa multi-cloud: estrategias de portabilidad, vendor lock-in y abstracción de recursos</t>
+          <t>State management: local vs remote state, state locking, backends (S3, GCS, Azure Blob) y workspaces</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3299,7 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Fundamentos de IaC: filosofía declarativa vs imperativa, idempotencia y drift detection</t>
+          <t>Módulos: diseño, versionado, registro público y privado, composición y reusabilidad</t>
         </is>
       </c>
     </row>
@@ -3278,7 +3316,7 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>HCL: sintaxis, tipos de datos, expresiones, funciones y meta-argumentos (count, for_each, depends_on)</t>
+          <t>Patrones avanzados: for_each, dynamic blocks, moved blocks, import y workspaces</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3333,7 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Providers: configuración, autenticación y uso de los providers de AWS, Azure y GCP</t>
+          <t>Terraform en CI/CD: plan/apply automatizado, Atlantis y GitHub Actions</t>
         </is>
       </c>
     </row>
@@ -3312,7 +3350,7 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>State management: local vs remote state, state locking, backends (S3, GCS, Azure Blob) y workspaces</t>
+          <t>Testing de infraestructura: terraform test, tflint, checkov, tfsec y políticas con OPA/Conftest</t>
         </is>
       </c>
     </row>
@@ -3329,75 +3367,75 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Módulos: diseño, versionado, registro público y privado, composición y reusabilidad</t>
+          <t>Alternativas complementarias: OpenTofu, Pulumi y CDKTF</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura como Código con Terraform</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>Patrones avanzados: for_each, dynamic blocks, moved blocks, import y workspaces</t>
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Contenedores y Ecosistema OCI</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Arquitectura de contenedores: Linux namespaces, cgroups v2, UnionFS y el modelo de capas OCI</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura como Código con Terraform</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>Terraform en CI/CD: plan/apply automatizado, Atlantis y GitHub Actions</t>
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Contenedores y Ecosistema OCI</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Dockerfile avanzado: multi-stage builds, BuildKit, cache optimization y distroless/scratch images</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura como Código con Terraform</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>Testing de infraestructura: terraform test, tflint, checkov, tfsec y políticas con OPA/Conftest</t>
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Contenedores y Ecosistema OCI</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Container runtimes: Docker, containerd, CRI-O, runc, gVisor y la interfaz CRI de Kubernetes</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura como Código con Terraform</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>Alternativas complementarias: OpenTofu, Pulumi y CDKTF</t>
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Contenedores y Ecosistema OCI</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Docker Compose: definición de servicios multi-contenedor, redes, volúmenes y profiles</t>
         </is>
       </c>
     </row>
@@ -3414,7 +3452,7 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Arquitectura de contenedores: Linux namespaces, cgroups v2, UnionFS y el modelo de capas OCI</t>
+          <t>Registros de imágenes: Docker Hub, GHCR, ECR, ACR, GAR y Harbor como registro privado</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3469,7 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Dockerfile avanzado: multi-stage builds, BuildKit, cache optimization y distroless/scratch images</t>
+          <t>Seguridad de imágenes: CVE scanning con Trivy/Grype, image signing con Cosign y generación de SBOM</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3486,7 @@
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Container runtimes: Docker, containerd, CRI-O, runc, gVisor y la interfaz CRI de Kubernetes</t>
+          <t>Builds in-cluster: kaniko, buildah y Paketo Buildpacks para entornos sin Docker daemon</t>
         </is>
       </c>
     </row>
@@ -3465,7 +3503,7 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Docker Compose: definición de servicios multi-contenedor, redes, volúmenes y profiles</t>
+          <t>Optimización: reducción de tamaño, gestión de capas, secrets en build time y multi-platform builds</t>
         </is>
       </c>
     </row>
@@ -3482,7 +3520,7 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Registros de imágenes: Docker Hub, GHCR, ECR, ACR, GAR y Harbor como registro privado</t>
+          <t>OCI Artifacts: almacenamiento de Helm charts, políticas OPA y otros artefactos en registros OCI</t>
         </is>
       </c>
     </row>
@@ -3494,12 +3532,12 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Contenedores y Ecosistema OCI</t>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Seguridad de imágenes: CVE scanning con Trivy/Grype, image signing con Cosign y generación de SBOM</t>
+          <t>Introducción · Control Plane: kube-apiserver, etcd, kube-scheduler, controller-manager, cloud-controller-manager</t>
         </is>
       </c>
     </row>
@@ -3511,12 +3549,12 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Contenedores y Ecosistema OCI</t>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Builds in-cluster: kaniko, buildah y Paketo Buildpacks para entornos sin Docker daemon</t>
+          <t>Introducción · Data Plane: kubelet, kube-proxy, container runtime y comunicación entre nodos</t>
         </is>
       </c>
     </row>
@@ -3528,12 +3566,12 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Contenedores y Ecosistema OCI</t>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Optimización: reducción de tamaño, gestión de capas, secrets en build time y multi-platform builds</t>
+          <t>Clusters locales · kind (Kubernetes in Docker): configuración multi-nodo, networking y uso en CI</t>
         </is>
       </c>
     </row>
@@ -3545,12 +3583,12 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Contenedores y Ecosistema OCI</t>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>OCI Artifacts: almacenamiento de Helm charts, políticas OPA y otros artefactos en registros OCI</t>
+          <t>Building Blocks · Pods: ciclo de vida, init containers, sidecar pattern y ephemeral containers</t>
         </is>
       </c>
     </row>
@@ -3567,7 +3605,7 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Introducción · Control Plane: kube-apiserver, etcd, kube-scheduler, controller-manager, cloud-controller-manager</t>
+          <t>Building Blocks · Workloads: Deployment, StatefulSet, DaemonSet, Job, CronJob y ReplicaSet</t>
         </is>
       </c>
     </row>
@@ -3584,7 +3622,7 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Introducción · Data Plane: kubelet, kube-proxy, container runtime y comunicación entre nodos</t>
+          <t>Building Blocks · Configuración: ConfigMap, Secret (tipos, encriptación at rest), env vars y volúmenes</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3639,7 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Clusters locales · kind (Kubernetes in Docker): configuración multi-nodo, networking y uso en CI</t>
+          <t>Building Blocks · Namespace, Labels, Selectors, Annotations, Finalizers y OwnerReferences</t>
         </is>
       </c>
     </row>
@@ -3618,7 +3656,7 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Building Blocks · Pods: ciclo de vida, init containers, sidecar pattern y ephemeral containers</t>
+          <t>Building Blocks · Scheduling: node/pod affinity, taints, tolerations, topology spread y priority classes</t>
         </is>
       </c>
     </row>
@@ -3635,7 +3673,7 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Building Blocks · Workloads: Deployment, StatefulSet, DaemonSet, Job, CronJob y ReplicaSet</t>
+          <t>Building Blocks · Resource management: requests, limits, LimitRange, ResourceQuota y QoS classes</t>
         </is>
       </c>
     </row>
@@ -3652,7 +3690,7 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Building Blocks · Configuración: ConfigMap, Secret (tipos, encriptación at rest), env vars y volúmenes</t>
+          <t>Almacenamiento · PersistentVolume, PersistentVolumeClaim, StorageClass, dynamic provisioning y CSI (EBS, Azure Disk, GCE PD)</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3707,7 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Building Blocks · Namespace, Labels, Selectors, Annotations, Finalizers y OwnerReferences</t>
+          <t>Networking · Services (ClusterIP, NodePort, LoadBalancer, Headless), Ingress, Gateway API, CNI (Calico, Cilium) y NetworkPolicy</t>
         </is>
       </c>
     </row>
@@ -3686,7 +3724,7 @@
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Building Blocks · Scheduling: node/pod affinity, taints, tolerations, topology spread y priority classes</t>
+          <t>Networking · DNS interno: CoreDNS, resolución de servicios y customización de zonas</t>
         </is>
       </c>
     </row>
@@ -3703,7 +3741,7 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Building Blocks · Resource management: requests, limits, LimitRange, ResourceQuota y QoS classes</t>
+          <t>Autenticación · RBAC: ServiceAccounts, Roles, ClusterRoles, Bindings y principio de mínimo privilegio</t>
         </is>
       </c>
     </row>
@@ -3720,7 +3758,7 @@
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Almacenamiento · PersistentVolume, PersistentVolumeClaim, StorageClass, dynamic provisioning y CSI (EBS, Azure Disk, GCE PD)</t>
+          <t>Autenticación · certificados X.509, OIDC, webhook auth, bound SA tokens y admission controllers (Gatekeeper, Kyverno, PSA)</t>
         </is>
       </c>
     </row>
@@ -3737,75 +3775,75 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Networking · Services (ClusterIP, NodePort, LoadBalancer, Headless), Ingress, Gateway API, CNI (Calico, Cilium) y NetworkPolicy</t>
+          <t>Cluster desde cero · etcd, kube-apiserver, scheduler, controller-manager, kubelet, kube-proxy: configuración manual, PKI y TLS bootstrapping</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B82" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>Networking · DNS interno: CoreDNS, resolución de servicios y customización de zonas</t>
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>EKS (AWS): arquitectura, node groups (managed, self-managed, Fargate), eksctl</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B83" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C83" s="5" t="inlineStr">
-        <is>
-          <t>Autenticación · RBAC: ServiceAccounts, Roles, ClusterRoles, Bindings y principio de mínimo privilegio</t>
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>EKS Add-ons: AWS Load Balancer Controller, EBS/EFS CSI, VPC CNI, ExternalDNS</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B84" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C84" s="5" t="inlineStr">
-        <is>
-          <t>Autenticación · certificados X.509, OIDC, webhook auth, bound SA tokens y admission controllers (Gatekeeper, Kyverno, PSA)</t>
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>EKS Seguridad: IRSA, EKS Pod Identity, KMS encryption y audit logging</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B85" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C85" s="5" t="inlineStr">
-        <is>
-          <t>Cluster desde cero · etcd, kube-apiserver, scheduler, controller-manager, kubelet, kube-proxy: configuración manual, PKI y TLS bootstrapping</t>
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>GKE: Standard vs Autopilot, node pools, Workload Identity y VPC-native networking</t>
         </is>
       </c>
     </row>
@@ -3822,7 +3860,7 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>EKS (AWS): arquitectura, node groups (managed, self-managed, Fargate), eksctl</t>
+          <t>GKE Add-ons: Cloud Operations, Config Connector, GKE Gateway y Fleet Management</t>
         </is>
       </c>
     </row>
@@ -3839,7 +3877,7 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>EKS Add-ons: AWS Load Balancer Controller, EBS/EFS CSI, VPC CNI, ExternalDNS</t>
+          <t>AKS: arquitectura, AAD/Entra ID integration, Managed Identities y Azure CNI</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3894,7 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>EKS Seguridad: IRSA, EKS Pod Identity, KMS encryption y audit logging</t>
+          <t>AKS Add-ons: Azure Monitor, CSI drivers (Disk/Files/Blob), AGIC y Azure Policy</t>
         </is>
       </c>
     </row>
@@ -3873,7 +3911,7 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>GKE: Standard vs Autopilot, node pools, Workload Identity y VPC-native networking</t>
+          <t>AKS Seguridad: Workload Identity, Azure Key Vault CSI Provider y Defender for Containers</t>
         </is>
       </c>
     </row>
@@ -3890,7 +3928,7 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>GKE Add-ons: Cloud Operations, Config Connector, GKE Gateway y Fleet Management</t>
+          <t>Otros entornos: OVHcloud, DigitalOcean DOKS, Linode LKE, on-premises (k3s, k0s, Rancher, OpenShift)</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3945,7 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>AKS: arquitectura, AAD/Entra ID integration, Managed Identities y Azure CNI</t>
+          <t>Aprovisionamiento IaC: Terraform modules para EKS, GKE y AKS. Comparativa multi-cloud</t>
         </is>
       </c>
     </row>
@@ -3919,12 +3957,12 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
+          <t>Application Bundles e Infraestructura Declarativa</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>AKS Add-ons: Azure Monitor, CSI drivers (Disk/Files/Blob), AGIC y Azure Policy</t>
+          <t>Kustomize: bases, overlays, patches, generators y transformers. 2 ejemplos prácticos (dev/prod)</t>
         </is>
       </c>
     </row>
@@ -3936,12 +3974,12 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
+          <t>Application Bundles e Infraestructura Declarativa</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>AKS Seguridad: Workload Identity, Azure Key Vault CSI Provider y Defender for Containers</t>
+          <t>Helm: charts, templates, values, hooks. El catálogo de Helm (Artifact Hub) como ecosistema de distribución</t>
         </is>
       </c>
     </row>
@@ -3953,12 +3991,12 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
+          <t>Application Bundles e Infraestructura Declarativa</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Otros entornos: OVHcloud, DigitalOcean DOKS, Linode LKE, on-premises (k3s, k0s, Rancher, OpenShift)</t>
+          <t>Helm + Kustomize: helm-secrets, helm-diff. Combinar render de Helm con overlays Kustomize por entorno</t>
         </is>
       </c>
     </row>
@@ -3970,12 +4008,12 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
+          <t>Application Bundles e Infraestructura Declarativa</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Aprovisionamiento IaC: Terraform modules para EKS, GKE y AKS. Comparativa multi-cloud</t>
+          <t>Caso real: charts que despliegan operators (kube-prometheus-stack, Grafana Operator). Se profundiza en la Sesión 24</t>
         </is>
       </c>
     </row>
@@ -3992,7 +4030,7 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Helm: charts, templates, values, hooks, repositorios, helm-secrets y helm-diff</t>
+          <t>ExternalDNS: providers (Route53, CloudDNS, Cloudflare), anotaciones y políticas de sync</t>
         </is>
       </c>
     </row>
@@ -4009,7 +4047,7 @@
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>Kustomize: bases, overlays, patches, generators y transformers. Helm + Kustomize</t>
+          <t>cert-manager: Issuers, ClusterIssuers, Let's Encrypt, ACME DNS-01/HTTP-01, renovación automática</t>
         </is>
       </c>
     </row>
@@ -4026,7 +4064,7 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>Patrón Operator: CRDs, controller loop, Operator Lifecycle Manager, niveles de madurez</t>
+          <t>Crossplane: Providers, Managed Resources, Compositions, XRDs. Comparativa con Terraform</t>
         </is>
       </c>
     </row>
@@ -4043,7 +4081,7 @@
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Operators de referencia: cert-manager, Prometheus Operator, Strimzi, Crossplane</t>
+          <t>Crossplane avanzado: Composition Functions, EnvironmentConfigs, integración con ArgoCD</t>
         </is>
       </c>
     </row>
@@ -4055,12 +4093,12 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>Application Bundles e Infraestructura Declarativa</t>
+          <t>Gestión de Secretos: Vault y External Secrets</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>ExternalDNS: providers (Route53, CloudDNS, Cloudflare), anotaciones y políticas de sync</t>
+          <t>Vault · Arquitectura: server, agents, backends de almacenamiento y alta disponibilidad</t>
         </is>
       </c>
     </row>
@@ -4072,12 +4110,12 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Application Bundles e Infraestructura Declarativa</t>
+          <t>Gestión de Secretos: Vault y External Secrets</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>cert-manager: Issuers, ClusterIssuers, Let's Encrypt, ACME DNS-01/HTTP-01, renovación automática</t>
+          <t>Vault · Auth methods en Kubernetes: Kubernetes Auth, JWT/OIDC, AppRole y cloud IAM</t>
         </is>
       </c>
     </row>
@@ -4089,12 +4127,12 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Application Bundles e Infraestructura Declarativa</t>
+          <t>Gestión de Secretos: Vault y External Secrets</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>Crossplane: Providers, Managed Resources, Compositions, XRDs. Comparativa con Terraform</t>
+          <t>Vault · Secrets Engines: KV v1/v2, Dynamic Secrets (database, AWS, Azure), PKI y Transit</t>
         </is>
       </c>
     </row>
@@ -4106,12 +4144,12 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Application Bundles e Infraestructura Declarativa</t>
+          <t>Gestión de Secretos: Vault y External Secrets</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>Crossplane avanzado: Composition Functions, EnvironmentConfigs, integración con ArgoCD</t>
+          <t>Vault · Vault Agent: auto-auth, template rendering, sidecar injection. Vault Secrets Operator (VSO)</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4166,7 @@
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Vault · Arquitectura: server, agents, backends de almacenamiento y alta disponibilidad</t>
+          <t>Vault · Políticas (HCL), namespaces, auditing, DR con Raft y auto-unseal con KMS (AWS, Azure, GCP)</t>
         </is>
       </c>
     </row>
@@ -4145,7 +4183,7 @@
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Vault · Auth methods en Kubernetes: Kubernetes Auth, JWT/OIDC, AppRole y cloud IAM</t>
+          <t>External Secrets · ExternalSecret, SecretStore, ClusterSecretStore y refresh intervals</t>
         </is>
       </c>
     </row>
@@ -4162,7 +4200,7 @@
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>Vault · Secrets Engines: KV v1/v2, Dynamic Secrets (database, AWS, Azure), PKI y Transit</t>
+          <t>External Secrets · Providers: AWS Secrets Manager, Azure Key Vault, GCP Secret Manager y Vault</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4217,7 @@
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Vault · Vault Agent: auto-auth, template rendering, sidecar injection. Vault Secrets Operator (VSO)</t>
+          <t>External Secrets · Patrones avanzados: secret templating, generators, pushSecret e integración con GitOps</t>
         </is>
       </c>
     </row>
@@ -4196,75 +4234,75 @@
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>Vault · Políticas (HCL), namespaces, auditing, DR con Raft y auto-unseal con KMS (AWS, Azure, GCP)</t>
+          <t>Secret Management · Sealed Secrets, SOPS y comparativa de patrones por madurez</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B109" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Secretos: Vault y External Secrets</t>
-        </is>
-      </c>
-      <c r="C109" s="3" t="inlineStr">
-        <is>
-          <t>External Secrets · ExternalSecret, SecretStore, ClusterSecretStore y refresh intervals</t>
+      <c r="A109" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>Observabilidad (I): Métricas</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>Los tres pilares: métricas, logs, trazas. Correlación entre señales</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B110" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Secretos: Vault y External Secrets</t>
-        </is>
-      </c>
-      <c r="C110" s="3" t="inlineStr">
-        <is>
-          <t>External Secrets · Providers: AWS Secrets Manager, Azure Key Vault, GCP Secret Manager y Vault</t>
+      <c r="A110" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>Observabilidad (I): Métricas</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>Prometheus: arquitectura, scraping, PromQL, service discovery, Alertmanager</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B111" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Secretos: Vault y External Secrets</t>
-        </is>
-      </c>
-      <c r="C111" s="3" t="inlineStr">
-        <is>
-          <t>External Secrets · Patrones avanzados: secret templating, generators, pushSecret e integración con GitOps</t>
+      <c r="A111" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>Observabilidad (I): Métricas</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>Prometheus Operator: ServiceMonitor, PodMonitor, recording rules, alerting rules. Thanos para HA</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B112" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Secretos: Vault y External Secrets</t>
-        </is>
-      </c>
-      <c r="C112" s="3" t="inlineStr">
-        <is>
-          <t>Secret Management · Sealed Secrets, SOPS y comparativa de patrones por madurez</t>
+      <c r="A112" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>Observabilidad (II): Grafana y Logs</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>Grafana: datasources, dashboards, variables, alerting. Grafana as Code (grafonnet, Terraform)</t>
         </is>
       </c>
     </row>
@@ -4276,12 +4314,12 @@
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>Observabilidad</t>
+          <t>Observabilidad (II): Grafana y Logs</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Los tres pilares: métricas, logs, trazas. Correlación entre señales</t>
+          <t>Loki: arquitectura, LogQL (mismo modelo mental que PromQL), labels vs indexación de texto completo</t>
         </is>
       </c>
     </row>
@@ -4293,12 +4331,12 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>Observabilidad</t>
+          <t>Observabilidad (II): Grafana y Logs</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>Prometheus: arquitectura, scraping, PromQL, service discovery, Alertmanager</t>
+          <t>Promtail: recolección de logs de los Pods y envío a Loki</t>
         </is>
       </c>
     </row>
@@ -4310,12 +4348,12 @@
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>Observabilidad</t>
+          <t>Observabilidad (II): Grafana y Logs</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Prometheus Operator: ServiceMonitor, PodMonitor, recording rules, alerting rules. Thanos para HA</t>
+          <t>Grafana Explore: consulta y filtrado de logs por label en tiempo real</t>
         </is>
       </c>
     </row>
@@ -4327,12 +4365,12 @@
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>Observabilidad</t>
+          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>Grafana: datasources, dashboards, variables, alerting. Grafana as Code (grafonnet, Terraform)</t>
+          <t>OpenTelemetry: especificación OTLP, SDK, auto-instrumentación de la app sin tocar código</t>
         </is>
       </c>
     </row>
@@ -4344,12 +4382,12 @@
       </c>
       <c r="B117" s="5" t="inlineStr">
         <is>
-          <t>Observabilidad</t>
+          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Grafana stack: Loki (logs), Tempo (trazas), Mimir (métricas), Alloy (collector)</t>
+          <t>OpenTelemetry Collector: pipeline de receivers, processors y exporters</t>
         </is>
       </c>
     </row>
@@ -4361,12 +4399,12 @@
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>Observabilidad</t>
+          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>OpenTelemetry: especificación OTLP, Collector pipelines, auto-instrumentación en Kubernetes</t>
+          <t>Tempo: backend de trazas distribuidas, trace ID, spans, integración con Grafana</t>
         </is>
       </c>
     </row>
@@ -4378,12 +4416,12 @@
       </c>
       <c r="B119" s="5" t="inlineStr">
         <is>
-          <t>Observabilidad</t>
+          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Stack completo: Prometheus + Grafana + Loki + Tempo + OTel Collector integrados</t>
+          <t>Mimir: métricas a escala/federadas (mención breve, complementa Prometheus de la Sesión 19)</t>
         </is>
       </c>
     </row>
@@ -4395,12 +4433,12 @@
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>GitOps y Pipelines CI/CD</t>
+          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>Principios GitOps: declarativo, versionado, automatizado, reconciliado. Pull vs Push model</t>
+          <t>Correlación end-to-end: exemplars, salto métrica→traza→logs en un mismo dashboard</t>
         </is>
       </c>
     </row>
@@ -4417,7 +4455,7 @@
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>ArgoCD: Applications, AppProjects, ApplicationSets, sync policies, waves, hooks y RBAC</t>
+          <t>Principios GitOps: declarativo, versionado, automatizado, reconciliado. Pull vs Push model</t>
         </is>
       </c>
     </row>
@@ -4434,7 +4472,7 @@
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>ArgoCD avanzado: multi-tenancy, SSO, App of Apps, ApplicationSet generators y notifications</t>
+          <t>ArgoCD: Applications, AppProjects, ApplicationSets, sync policies, waves, hooks y RBAC</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4489,7 @@
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>ArgoCD Image Updater y Argo Rollouts: patrones de Progressive Delivery con análisis automático</t>
+          <t>ArgoCD avanzado: multi-tenancy, SSO, App of Apps, ApplicationSet generators y notifications</t>
         </is>
       </c>
     </row>
@@ -4468,7 +4506,7 @@
       </c>
       <c r="C124" s="5" t="inlineStr">
         <is>
-          <t>Prow: arquitectura CI nativa en Kubernetes, plugins, Tide, Deck dashboard y ProwJobs</t>
+          <t>ArgoCD Image Updater y Argo Rollouts: patrones de Progressive Delivery con análisis automático</t>
         </is>
       </c>
     </row>
@@ -4485,7 +4523,7 @@
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Tekton: Tasks, Pipelines, PipelineRuns, Workspaces, Triggers y Tekton Chains</t>
+          <t>Prow: arquitectura CI nativa en Kubernetes, plugins, Tide, Deck dashboard y ProwJobs</t>
         </is>
       </c>
     </row>
@@ -4502,7 +4540,7 @@
       </c>
       <c r="C126" s="5" t="inlineStr">
         <is>
-          <t>Integración Tekton + ArgoCD para workflows CI/CD end-to-end en Kubernetes</t>
+          <t>Tekton: Tasks, Pipelines, PipelineRuns, Workspaces, Triggers y Tekton Chains</t>
         </is>
       </c>
     </row>
@@ -4514,12 +4552,12 @@
       </c>
       <c r="B127" s="5" t="inlineStr">
         <is>
-          <t>Networking Avanzado (Service Mesh)</t>
+          <t>GitOps y Pipelines CI/CD</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Traefik: IngressRoute CRDs, middlewares, TLS automático, dashboard y métricas</t>
+          <t>Integración Tekton + ArgoCD para workflows CI/CD end-to-end en Kubernetes</t>
         </is>
       </c>
     </row>
@@ -4536,7 +4574,7 @@
       </c>
       <c r="C128" s="5" t="inlineStr">
         <is>
-          <t>Traefik avanzado: TCP/UDP routing, rate limiting, circuit breaker, canary con TraefikService</t>
+          <t>Traefik: IngressRoute CRDs, middlewares, TLS automático, dashboard y métricas</t>
         </is>
       </c>
     </row>
@@ -4553,7 +4591,7 @@
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Istio: arquitectura (Istiod + Envoy sidecars), mTLS automático y observabilidad integrada</t>
+          <t>Traefik avanzado: TCP/UDP routing, rate limiting, circuit breaker, canary con TraefikService</t>
         </is>
       </c>
     </row>
@@ -4570,7 +4608,7 @@
       </c>
       <c r="C130" s="5" t="inlineStr">
         <is>
-          <t>Istio traffic: VirtualServices, DestinationRules, Gateways, traffic shifting, fault injection</t>
+          <t>Istio: arquitectura (Istiod + Envoy sidecars), mTLS automático y observabilidad integrada</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4625,7 @@
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>Istio seguridad: AuthorizationPolicies, PeerAuthentication, circuit breaking, Kiali</t>
+          <t>Istio traffic: VirtualServices, DestinationRules, Gateways, traffic shifting, fault injection</t>
         </is>
       </c>
     </row>
@@ -4604,7 +4642,7 @@
       </c>
       <c r="C132" s="5" t="inlineStr">
         <is>
-          <t>Ambient Mesh (Istio): modo sin sidecar, ztunnel, waypoints y migración</t>
+          <t>Istio seguridad: AuthorizationPolicies, PeerAuthentication, circuit breaking, Kiali</t>
         </is>
       </c>
     </row>
@@ -4616,12 +4654,12 @@
       </c>
       <c r="B133" s="5" t="inlineStr">
         <is>
-          <t>Entrega Progresiva y Escalado</t>
+          <t>Networking Avanzado (Service Mesh)</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>Estrategias: rolling update, blue/green, canary, A/B testing y trade-offs</t>
+          <t>Ambient Mesh (Istio): modo sin sidecar, ztunnel, waypoints y migración</t>
         </is>
       </c>
     </row>
@@ -4638,7 +4676,7 @@
       </c>
       <c r="C134" s="5" t="inlineStr">
         <is>
-          <t>Argo Rollouts: canary con análisis automatizado, blue-green, integración Istio/Traefik + Prometheus</t>
+          <t>Estrategias: rolling update, blue/green, canary, A/B testing y trade-offs</t>
         </is>
       </c>
     </row>
@@ -4655,7 +4693,7 @@
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>Progressive delivery: Feature flags (Flagger/OpenFeature), métricas como gates, rollback automático</t>
+          <t>Argo Rollouts: canary con análisis automatizado, blue-green, integración Istio/Traefik + Prometheus</t>
         </is>
       </c>
     </row>
@@ -4672,7 +4710,7 @@
       </c>
       <c r="C136" s="5" t="inlineStr">
         <is>
-          <t>HPA: métricas CPU/memory, custom metrics (Prometheus Adapter), scaling behavior</t>
+          <t>Progressive delivery: Feature flags (Flagger/OpenFeature), métricas como gates, rollback automático</t>
         </is>
       </c>
     </row>
@@ -4689,7 +4727,7 @@
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>VPA: modos (Off/Initial/Auto), recomendaciones y limitaciones</t>
+          <t>HPA: métricas CPU/memory, custom metrics (Prometheus Adapter), scaling behavior</t>
         </is>
       </c>
     </row>
@@ -4706,7 +4744,7 @@
       </c>
       <c r="C138" s="5" t="inlineStr">
         <is>
-          <t>KEDA: ScaledObject, ScaledJob, triggers (Kafka, SQS, Prometheus, cron) y cooldown</t>
+          <t>VPA: modos (Off/Initial/Auto), recomendaciones y limitaciones</t>
         </is>
       </c>
     </row>
@@ -4723,24 +4761,24 @@
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
+          <t>KEDA: ScaledObject, ScaledJob, triggers (Kafka, SQS, Prometheus, cron) y cooldown</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B140" s="5" t="inlineStr">
+        <is>
+          <t>Entrega Progresiva y Escalado</t>
+        </is>
+      </c>
+      <c r="C140" s="5" t="inlineStr">
+        <is>
           <t>Cluster Autoscaler vs Karpenter: node pools, scale-from-zero, cost optimization</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B140" s="3" t="inlineStr">
-        <is>
-          <t>Construcción de Operators</t>
-        </is>
-      </c>
-      <c r="C140" s="3" t="inlineStr">
-        <is>
-          <t>Operator SDK (Go): scaffolding, CRD design, controller implementation y webhooks</t>
         </is>
       </c>
     </row>
@@ -4752,12 +4790,12 @@
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>Construcción de Operators</t>
+          <t>Go: de cero a controlador de Kubernetes</t>
         </is>
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>kubebuilder: reconciliation patterns, finalizers, status conditions y API versioning</t>
+          <t>Fundamentos de Go: tipos, structs, interfaces, goroutines, channels, manejo de errores idiomático</t>
         </is>
       </c>
     </row>
@@ -4769,12 +4807,12 @@
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>Construcción de Operators</t>
+          <t>Go: de cero a controlador de Kubernetes</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>Operadores de producción: leader election, metrics, testing (envtest) y OLM</t>
+          <t>client-go: clientset, kubeconfig, serialización, listar/filtrar/crear recursos de la API</t>
         </is>
       </c>
     </row>
@@ -4786,12 +4824,12 @@
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Clústeres y Serverless</t>
+          <t>Go: de cero a controlador de Kubernetes</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>Cluster API (CAPI): arquitectura, providers (AWS/Azure/GCP), lifecycle y upgrades</t>
+          <t>controller-runtime: reconciliation loop, informers, predicates (fundamentos, sin construir el operator todavía)</t>
         </is>
       </c>
     </row>
@@ -4803,12 +4841,12 @@
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Clústeres y Serverless</t>
+          <t>Go: de cero a controlador de Kubernetes</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
         <is>
-          <t>Rancher Fleet y ArgoCD ApplicationSets para gestión de flotas de clusters</t>
+          <t>CLIs y tooling: cobra/viper, logging estructurado, go test, mocks con testify, golangci-lint</t>
         </is>
       </c>
     </row>
@@ -4820,12 +4858,12 @@
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Clústeres y Serverless</t>
+          <t>Construcción de Operators</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>Upgrade strategies: rolling upgrades, ventanas de mantenimiento y node drain</t>
+          <t>Operator SDK (Go): scaffolding, CRD design, controller implementation y webhooks</t>
         </is>
       </c>
     </row>
@@ -4837,12 +4875,12 @@
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Clústeres y Serverless</t>
+          <t>Construcción de Operators</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
         <is>
-          <t>Knative Serving: auto-scaling a cero, revision routing y traffic splitting</t>
+          <t>kubebuilder: reconciliation patterns, finalizers, status conditions y API versioning</t>
         </is>
       </c>
     </row>
@@ -4854,12 +4892,12 @@
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Clústeres y Serverless</t>
+          <t>Construcción de Operators</t>
         </is>
       </c>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>Virtual Kubelet: nodos virtuales con Fargate, ACI y Cloud Run</t>
+          <t>Operadores de producción: leader election, metrics, testing (envtest) y OLM</t>
         </is>
       </c>
     </row>
@@ -4871,12 +4909,12 @@
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>Hosted Control Planes</t>
+          <t>Gestión de Clústeres y Serverless</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>HyperShift (Red Hat): arquitectura, hosted clusters y node pools</t>
+          <t>Cluster API (CAPI): arquitectura, providers (AWS/Azure/GCP), lifecycle y upgrades</t>
         </is>
       </c>
     </row>
@@ -4888,12 +4926,12 @@
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>Hosted Control Planes</t>
+          <t>Gestión de Clústeres y Serverless</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
-          <t>vCluster: clusters virtuales ligeros, sincronización y multi-tenancy</t>
+          <t>Rancher Fleet y ArgoCD ApplicationSets para gestión de flotas de clusters</t>
         </is>
       </c>
     </row>
@@ -4905,12 +4943,12 @@
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>Hosted Control Planes</t>
+          <t>Gestión de Clústeres y Serverless</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>Kamaji: tenant control planes, datastores y gestión de flota</t>
+          <t>Upgrade strategies: rolling upgrades, ventanas de mantenimiento y node drain</t>
         </is>
       </c>
     </row>
@@ -4922,12 +4960,12 @@
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>Multi-cluster y Multi-cloud</t>
+          <t>Gestión de Clústeres y Serverless</t>
         </is>
       </c>
       <c r="C151" s="3" t="inlineStr">
         <is>
-          <t>Arquitecturas: hub-and-spoke, peer-to-peer, federación</t>
+          <t>Knative Serving: auto-scaling a cero, revision routing y traffic splitting</t>
         </is>
       </c>
     </row>
@@ -4939,12 +4977,12 @@
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>Multi-cluster y Multi-cloud</t>
+          <t>Gestión de Clústeres y Serverless</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>Open Cluster Management (OCM), Rancher MCM y ArgoCD multicluster</t>
+          <t>Virtual Kubelet: nodos virtuales con Fargate, ACI y Cloud Run</t>
         </is>
       </c>
     </row>
@@ -4956,12 +4994,12 @@
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>Multi-cluster y Multi-cloud</t>
+          <t>Hosted Control Planes</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>Istio multicluster (primary-remote, multi-primary)</t>
+          <t>HyperShift (Red Hat): arquitectura, hosted clusters y node pools</t>
         </is>
       </c>
     </row>
@@ -4973,12 +5011,12 @@
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>Multi-cluster y Multi-cloud</t>
+          <t>Hosted Control Planes</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>Cilium Cluster Mesh: tunneling, shared services y network policies globales</t>
+          <t>vCluster: clusters virtuales ligeros, sincronización y multi-tenancy</t>
         </is>
       </c>
     </row>
@@ -4990,12 +5028,12 @@
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>Multi-cluster y Multi-cloud</t>
+          <t>Hosted Control Planes</t>
         </is>
       </c>
       <c r="C155" s="3" t="inlineStr">
         <is>
-          <t>Submariner: cross-cluster networking, service discovery y globalnet</t>
+          <t>Kamaji: tenant control planes, datastores y gestión de flota</t>
         </is>
       </c>
     </row>
@@ -5012,7 +5050,7 @@
       </c>
       <c r="C156" s="3" t="inlineStr">
         <is>
-          <t>Crossplane como plano de control universal, políticas OPA y ESO multi-cloud</t>
+          <t>Arquitecturas: hub-and-spoke, peer-to-peer, federación</t>
         </is>
       </c>
     </row>
@@ -5029,92 +5067,92 @@
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
+          <t>Open Cluster Management (OCM), Rancher MCM y ArgoCD multicluster</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>Multi-cluster y Multi-cloud</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>Istio multicluster (primary-remote, multi-primary)</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>Multi-cluster y Multi-cloud</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>Cilium Cluster Mesh: tunneling, shared services y network policies globales</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>Multi-cluster y Multi-cloud</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>Submariner: cross-cluster networking, service discovery y globalnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>Multi-cluster y Multi-cloud</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>Crossplane como plano de control universal, políticas OPA y ESO multi-cloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>Multi-cluster y Multi-cloud</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
           <t>Disaster Recovery: Velero, replicación de estado, RPO/RTO y failover automático</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="8" t="inlineStr">
-        <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="B158" s="5" t="inlineStr">
-        <is>
-          <t>Plataforma Interna de Desarrollo end-to-end</t>
-        </is>
-      </c>
-      <c r="C158" s="5" t="inlineStr">
-        <is>
-          <t>Aprovisionamiento de la infraestructura base con Terraform sobre uno o varios proveedores cloud</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="8" t="inlineStr">
-        <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="B159" s="5" t="inlineStr">
-        <is>
-          <t>Plataforma Interna de Desarrollo end-to-end</t>
-        </is>
-      </c>
-      <c r="C159" s="5" t="inlineStr">
-        <is>
-          <t>Despliegue y configuración de un clúster Kubernetes gestionado</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="8" t="inlineStr">
-        <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="B160" s="5" t="inlineStr">
-        <is>
-          <t>Plataforma Interna de Desarrollo end-to-end</t>
-        </is>
-      </c>
-      <c r="C160" s="5" t="inlineStr">
-        <is>
-          <t>Flujo GitOps con ArgoCD para el ciclo de vida de las aplicaciones de plataforma</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="8" t="inlineStr">
-        <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="B161" s="5" t="inlineStr">
-        <is>
-          <t>Plataforma Interna de Desarrollo end-to-end</t>
-        </is>
-      </c>
-      <c r="C161" s="5" t="inlineStr">
-        <is>
-          <t>Gestión de secretos con Vault y/o External Secrets Operator</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="8" t="inlineStr">
-        <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="B162" s="5" t="inlineStr">
-        <is>
-          <t>Plataforma Interna de Desarrollo end-to-end</t>
-        </is>
-      </c>
-      <c r="C162" s="5" t="inlineStr">
-        <is>
-          <t>Stack de observabilidad (métricas, logs, trazas) y alerting</t>
         </is>
       </c>
     </row>
@@ -5131,7 +5169,7 @@
       </c>
       <c r="C163" s="5" t="inlineStr">
         <is>
-          <t>Entrega progresiva (canary o blue/green) con rollback automático basado en métricas</t>
+          <t>Aprovisionamiento de la infraestructura base con Terraform sobre uno o varios proveedores cloud</t>
         </is>
       </c>
     </row>
@@ -5147,6 +5185,91 @@
         </is>
       </c>
       <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>Despliegue y configuración de un clúster Kubernetes gestionado</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="8" t="inlineStr">
+        <is>
+          <t>PF</t>
+        </is>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>Plataforma Interna de Desarrollo end-to-end</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>Flujo GitOps con ArgoCD para el ciclo de vida de las aplicaciones de plataforma</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="8" t="inlineStr">
+        <is>
+          <t>PF</t>
+        </is>
+      </c>
+      <c r="B166" s="5" t="inlineStr">
+        <is>
+          <t>Plataforma Interna de Desarrollo end-to-end</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>Gestión de secretos con Vault y/o External Secrets Operator</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="8" t="inlineStr">
+        <is>
+          <t>PF</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>Plataforma Interna de Desarrollo end-to-end</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>Stack de observabilidad (métricas, logs, trazas) y alerting</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="8" t="inlineStr">
+        <is>
+          <t>PF</t>
+        </is>
+      </c>
+      <c r="B168" s="5" t="inlineStr">
+        <is>
+          <t>Plataforma Interna de Desarrollo end-to-end</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>Entrega progresiva (canary o blue/green) con rollback automático basado en métricas</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="8" t="inlineStr">
+        <is>
+          <t>PF</t>
+        </is>
+      </c>
+      <c r="B169" s="5" t="inlineStr">
+        <is>
+          <t>Plataforma Interna de Desarrollo end-to-end</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
         <is>
           <t>Documentación, golden paths y defensa del proyecto</t>
         </is>

</xml_diff>

<commit_message>
Sincronizar documentos y registrar posible ampliación de IaC
</commit_message>
<xml_diff>
--- a/Calendario_Postgrado_Kubernetes.xlsx
+++ b/Calendario_Postgrado_Kubernetes.xlsx
@@ -859,7 +859,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Redes, DNS y CDN con Cloudflare</t>
+          <t>AWS y fundamentos de Terraform/OpenTofu</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Control de versiones avanzado con Git</t>
+          <t>Azure e IaC: equivalencias y módulos</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
+          <t>GCP e IaC: estado y comparativa multicloud</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -974,12 +974,12 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Infraestructura como Código con Terraform</t>
+          <t>Contenedores y ecosistema OCI: imágenes, runtimes y seguridad</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Contenedores y ecosistema OCI: imágenes, runtimes y seguridad</t>
+          <t>Kubernetes: arquitectura, control plane y clusters locales (kind)</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Kubernetes: arquitectura, control plane y clusters locales (kind)</t>
+          <t>Building Blocks: workloads, configuración y scheduling</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Building Blocks: workloads, configuración y scheduling</t>
+          <t>Almacenamiento y networking en Kubernetes</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Almacenamiento y networking en Kubernetes</t>
+          <t>Autenticación, RBAC y clúster componente a componente</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
@@ -1174,12 +1174,12 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Autenticación, RBAC y clúster componente a componente</t>
+          <t>Kubernetes gestionado: EKS, GKE y AKS</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Kubernetes gestionado: EKS, GKE y AKS</t>
+          <t>Otros entornos y aprovisionamiento IaC multi-cloud</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Otros entornos y aprovisionamiento IaC multi-cloud</t>
+          <t>Application bundles: Kustomize, Helm y su ecosistema</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Application bundles: Kustomize, Helm y su ecosistema</t>
+          <t>Infraestructura declarativa: ExternalDNS, cert-manager y Crossplane</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura declarativa: ExternalDNS, cert-manager y Crossplane</t>
+          <t>Gestión de secretos: Vault y External Secrets Operator</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -1374,12 +1374,12 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Gestión de secretos: Vault y External Secrets Operator</t>
+          <t>Observabilidad (I): Prometheus, PromQL y Alertmanager</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Observabilidad (I): Prometheus, PromQL y Alertmanager</t>
+          <t>Observabilidad (II): Grafana y Loki (logs)</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Observabilidad (II): Grafana y Loki (logs)</t>
+          <t>Observabilidad (III): OpenTelemetry, Tempo y correlación</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Observabilidad (III): OpenTelemetry, Tempo y correlación</t>
+          <t>Git y GitOps con ArgoCD</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>GitOps y pipelines CI/CD: ArgoCD, Prow y Tekton</t>
+          <t>Pipelines CI/CD: Prow y Tekton</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
@@ -2220,12 +2220,12 @@
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>12h</t>
+          <t>9h</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Redes, DNS y CDN con Cloudflare · Control de Versiones Avanzado con Git · Cloud Computing: AWS, Azure y GCP · Infraestructura como Código con Terraform</t>
+          <t>AWS y fundamentos de Terraform/OpenTofu · Azure e IaC: equivalencias y módulos · GCP e IaC: estado y comparativa multicloud</t>
         </is>
       </c>
     </row>
@@ -2301,12 +2301,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>18h</t>
+          <t>21h</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Observabilidad (I): Métricas · Observabilidad (II): Grafana y Logs · Observabilidad (III): OpenTelemetry, Tempo y Correlación · GitOps y Pipelines CI/CD · Networking Avanzado (Service Mesh) · Entrega Progresiva y Escalado</t>
+          <t>Observabilidad (I): Métricas · Observabilidad (II): Grafana y Logs · Observabilidad (III): OpenTelemetry, Tempo y Correlación · Git y GitOps con ArgoCD · Pipelines CI/CD: Prow y Tekton · Networking Avanzado (Service Mesh) · Entrega Progresiva y Escalado</t>
         </is>
       </c>
     </row>
@@ -2394,7 +2394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C169"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2682,12 +2682,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Redes, DNS y CDN con Cloudflare</t>
+          <t>AWS y fundamentos de Terraform/OpenTofu</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Revisión de fundamentos TCP/IP, UDP, TLS 1.3/mTLS, HTTP/2 y HTTP/3 (QUIC)</t>
+          <t>AWS: IAM, regiones y zonas, VPC, subredes, Security Groups, EC2 y S3; contexto de ECR</t>
         </is>
       </c>
     </row>
@@ -2699,12 +2699,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Redes, DNS y CDN con Cloudflare</t>
+          <t>AWS y fundamentos de Terraform/OpenTofu</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>DNS: resolución recursiva e iterativa, registros (A, AAAA, CNAME, TXT, SRV, NS), TTL y propagación</t>
+          <t>Fundamentos IaC: declarativo, idempotencia y drift; Terraform/OpenTofu, HCL, provider y recursos</t>
         </is>
       </c>
     </row>
@@ -2716,12 +2716,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Redes, DNS y CDN con Cloudflare</t>
+          <t>AWS y fundamentos de Terraform/OpenTofu</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>DNS avanzado: DNSSEC, DNS-over-HTTPS, split-horizon DNS y service discovery basado en DNS</t>
+          <t>Caso práctico común: red, máquina virtual y almacenamiento; init, plan, apply y destroy; permisos y control de costes</t>
         </is>
       </c>
     </row>
@@ -2733,12 +2733,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Redes, DNS y CDN con Cloudflare</t>
+          <t>Azure e IaC: equivalencias y módulos</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>CDN: arquitectura, edge caching, routing geográfico, invalidación y cache-control headers</t>
+          <t>Azure: Entra ID, suscripciones, grupos de recursos, Managed Identities, VNet, NSG, máquinas virtuales y Blob Storage; contexto de ACR</t>
         </is>
       </c>
     </row>
@@ -2750,12 +2750,12 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Redes, DNS y CDN con Cloudflare</t>
+          <t>Azure e IaC: equivalencias y módulos</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Cloudflare: DNS authoritative, Cloudflare Tunnel, Workers, WAF, DDoS protection y R2</t>
+          <t>Transferencia del caso AWS a Azure con configuración preparada: equivalencias y diferencias</t>
         </is>
       </c>
     </row>
@@ -2767,12 +2767,12 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Redes, DNS y CDN con Cloudflare</t>
+          <t>Azure e IaC: equivalencias y módulos</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Certificados TLS: PKI, cadena de confianza, ACME protocol y automatización con Let's Encrypt</t>
+          <t>Terraform/OpenTofu: variables, outputs y uso de módulos existentes; sin diseño avanzado de módulos propios</t>
         </is>
       </c>
     </row>
@@ -2784,12 +2784,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Redes, DNS y CDN con Cloudflare</t>
+          <t>GCP e IaC: estado y comparativa multicloud</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Load balancing: algoritmos, health checks, session persistence y global load balancing</t>
+          <t>GCP: proyectos, cuentas de servicio, IAM, VPC, firewall, Compute Engine y Cloud Storage; contexto de Artifact Registry</t>
         </is>
       </c>
     </row>
@@ -2801,12 +2801,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Control de Versiones Avanzado con Git</t>
+          <t>GCP e IaC: estado y comparativa multicloud</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Arquitectura interna de Git: objects (blob, tree, commit, tag), refs, packfiles, reflog y garbage collection</t>
+          <t>Transferencia del mismo caso a GCP con configuración preparada; comparación de identidad, redes, permisos y portabilidad</t>
         </is>
       </c>
     </row>
@@ -2818,12 +2818,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Control de Versiones Avanzado con Git</t>
+          <t>GCP e IaC: estado y comparativa multicloud</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Estrategias de branching: Git Flow, GitHub Flow, trunk-based development y comparativa práctica</t>
+          <t>Terraform/OpenTofu: estado local y remoto, locking según backend y protección del estado y de las credenciales</t>
         </is>
       </c>
     </row>
@@ -2835,1406 +2835,1406 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Control de Versiones Avanzado con Git</t>
+          <t>GCP e IaC: estado y comparativa multicloud</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Rebases interactivos: squash, fixup, reword, edit y reordenación de commits</t>
+          <t>Pulumi: comparación de 10–15 minutos de HCL frente a Python/Go con un ejemplo equivalente pequeño; también requiere gestión de estado; sin instalación ni laboratorio propio</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Control de Versiones Avanzado con Git</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Resolución de conflictos: estrategias de merge (recursive, ort), rerere, git mergetool y best practices</t>
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Contenedores y Ecosistema OCI</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Arquitectura de contenedores: Linux namespaces, cgroups v2, UnionFS y el modelo de capas OCI</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Control de Versiones Avanzado con Git</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de ramas: naming conventions, branch protection rules, CODEOWNERS y cleanup automático</t>
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Contenedores y Ecosistema OCI</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Dockerfile avanzado: multi-stage builds, BuildKit, cache optimization y distroless/scratch images</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Control de Versiones Avanzado con Git</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Pull Requests y code review: merge strategies (merge, squash, rebase), signed commits y draft PRs</t>
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Contenedores y Ecosistema OCI</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Container runtimes: Docker, containerd, CRI-O, runc, gVisor y la interfaz CRI de Kubernetes</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>Control de Versiones Avanzado con Git</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Git hooks: pre-commit, commit-msg, post-merge y automatización con pre-commit framework</t>
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Contenedores y Ecosistema OCI</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Docker Compose: definición de servicios multi-contenedor, redes, volúmenes y profiles</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>Control de Versiones Avanzado con Git</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Monorepos: estrategias, herramientas (Nx, Turborepo) y gestión de dependencias</t>
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Contenedores y Ecosistema OCI</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Registros de imágenes: Docker Hub, GHCR, ECR, ACR, GAR y Harbor como registro privado</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>Control de Versiones Avanzado con Git</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Operaciones avanzadas: git bisect, git worktree, submodules, subtrees y sparse-checkout</t>
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Contenedores y Ecosistema OCI</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Seguridad de imágenes: CVE scanning con Trivy/Grype, image signing con Cosign y generación de SBOM</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>AWS · IAM: users, roles, policies, OIDC federation, IRSA y AWS SSO</t>
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Contenedores y Ecosistema OCI</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Builds in-cluster: kaniko, buildah y Paketo Buildpacks para entornos sin Docker daemon</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>AWS · Computación: EC2 (instance types, AMIs, user-data), Auto Scaling Groups, Lambda</t>
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Contenedores y Ecosistema OCI</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Optimización: reducción de tamaño, gestión de capas, secrets en build time y multi-platform builds</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>AWS · Redes: VPC, subnets públicas/privadas, Security Groups, ALB/NLB, Route 53 y PrivateLink</t>
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Contenedores y Ecosistema OCI</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>OCI Artifacts: almacenamiento de Helm charts, políticas OPA y otros artefactos en registros OCI</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>AWS · Almacenamiento: S3 (lifecycle, versioning), EBS, EFS y ECR</t>
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Introducción · Control Plane: kube-apiserver, etcd, kube-scheduler, controller-manager, cloud-controller-manager</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>AWS · Servicios gestionados: RDS, DynamoDB, SQS, CloudWatch y Secrets Manager</t>
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Introducción · Data Plane: kubelet, kube-proxy, container runtime y comunicación entre nodos</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>Azure · IAM: Entra ID, Managed Identities, RBAC y Azure Key Vault</t>
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Clusters locales · kind (Kubernetes in Docker): configuración multi-nodo, networking y uso en CI</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>Azure · Computación: VMs, VMSS, Azure Functions y Azure Container Apps</t>
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Building Blocks · Pods: ciclo de vida, init containers, sidecar pattern y ephemeral containers</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>Azure · Redes: VNet, subnets, NSG, Load Balancer, Application Gateway y Azure DNS</t>
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Building Blocks · Workloads: Deployment, StatefulSet, DaemonSet, Job, CronJob y ReplicaSet</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>Azure · Almacenamiento: Blob Storage, Azure Files, Managed Disks y ACR</t>
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Building Blocks · Configuración: ConfigMap, Secret (tipos, encriptación at rest), env vars y volúmenes</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>Azure · Servicios gestionados: Azure SQL, Cosmos DB, Service Bus y Azure Monitor</t>
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Building Blocks · Namespace, Labels, Selectors, Annotations, Finalizers y OwnerReferences</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>GCP · IAM: Service Accounts, Workload Identity, org policies y Cloud Audit Logs</t>
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Building Blocks · Scheduling: node/pod affinity, taints, tolerations, topology spread y priority classes</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>GCP · Computación: Compute Engine, Cloud Functions y Cloud Run</t>
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Building Blocks · Resource management: requests, limits, LimitRange, ResourceQuota y QoS classes</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>GCP · Redes: VPC, Firewall Rules, Cloud NAT, Cloud Load Balancing y Cloud DNS</t>
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Almacenamiento · PersistentVolume, PersistentVolumeClaim, StorageClass, dynamic provisioning y CSI (EBS, Azure Disk, GCE PD)</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>GCP · Almacenamiento: Cloud Storage, Persistent Disk y Artifact Registry</t>
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Networking · Services (ClusterIP, NodePort, LoadBalancer, Headless), Ingress, Gateway API, CNI (Calico, Cilium) y NetworkPolicy</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>GCP · Servicios gestionados: Cloud SQL, Firestore, Pub/Sub y Cloud Monitoring</t>
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Networking · DNS interno: CoreDNS, resolución de servicios y customización de zonas</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>Cloud Computing: AWS, Azure y GCP</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>Comparativa multi-cloud: estrategias de portabilidad, vendor lock-in y abstracción de recursos</t>
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Autenticación · RBAC: ServiceAccounts, Roles, ClusterRoles, Bindings y principio de mínimo privilegio</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura como Código con Terraform</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>Fundamentos de IaC: filosofía declarativa vs imperativa, idempotencia y drift detection</t>
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Autenticación · certificados X.509, OIDC, webhook auth, bound SA tokens y admission controllers (Gatekeeper, Kyverno, PSA)</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura como Código con Terraform</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>HCL: sintaxis, tipos de datos, expresiones, funciones y meta-argumentos (count, for_each, depends_on)</t>
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Cluster desde cero · etcd, kube-apiserver, scheduler, controller-manager, kubelet, kube-proxy: configuración manual, PKI y TLS bootstrapping</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura como Código con Terraform</t>
+          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Providers: configuración, autenticación y uso de los providers de AWS, Azure y GCP</t>
+          <t>EKS (AWS): arquitectura, node groups (managed, self-managed, Fargate), eksctl</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura como Código con Terraform</t>
+          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>State management: local vs remote state, state locking, backends (S3, GCS, Azure Blob) y workspaces</t>
+          <t>EKS Add-ons: AWS Load Balancer Controller, EBS/EFS CSI, VPC CNI, ExternalDNS</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura como Código con Terraform</t>
+          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Módulos: diseño, versionado, registro público y privado, composición y reusabilidad</t>
+          <t>EKS Seguridad: IRSA, EKS Pod Identity, KMS encryption y audit logging</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura como Código con Terraform</t>
+          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Patrones avanzados: for_each, dynamic blocks, moved blocks, import y workspaces</t>
+          <t>GKE: Standard vs Autopilot, node pools, Workload Identity y VPC-native networking</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura como Código con Terraform</t>
+          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Terraform en CI/CD: plan/apply automatizado, Atlantis y GitHub Actions</t>
+          <t>GKE Add-ons: Cloud Operations, Config Connector, GKE Gateway y Fleet Management</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura como Código con Terraform</t>
+          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Testing de infraestructura: terraform test, tflint, checkov, tfsec y políticas con OPA/Conftest</t>
+          <t>AKS: arquitectura, AAD/Entra ID integration, Managed Identities y Azure CNI</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura como Código con Terraform</t>
+          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Alternativas complementarias: OpenTofu, Pulumi y CDKTF</t>
+          <t>AKS Add-ons: Azure Monitor, CSI drivers (Disk/Files/Blob), AGIC y Azure Policy</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B58" s="5" t="inlineStr">
-        <is>
-          <t>Contenedores y Ecosistema OCI</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>Arquitectura de contenedores: Linux namespaces, cgroups v2, UnionFS y el modelo de capas OCI</t>
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>AKS Seguridad: Workload Identity, Azure Key Vault CSI Provider y Defender for Containers</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>Contenedores y Ecosistema OCI</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>Dockerfile avanzado: multi-stage builds, BuildKit, cache optimization y distroless/scratch images</t>
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Otros entornos: OVHcloud, DigitalOcean DOKS, Linode LKE, on-premises (k3s, k0s, Rancher, OpenShift)</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="inlineStr">
-        <is>
-          <t>Contenedores y Ecosistema OCI</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>Container runtimes: Docker, containerd, CRI-O, runc, gVisor y la interfaz CRI de Kubernetes</t>
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Aprovisionamiento IaC: Terraform modules para EKS, GKE y AKS. Comparativa multi-cloud</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B61" s="5" t="inlineStr">
-        <is>
-          <t>Contenedores y Ecosistema OCI</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>Docker Compose: definición de servicios multi-contenedor, redes, volúmenes y profiles</t>
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Application Bundles e Infraestructura Declarativa</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Kustomize: bases, overlays, patches, generators y transformers. 2 ejemplos prácticos (dev/prod)</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="inlineStr">
-        <is>
-          <t>Contenedores y Ecosistema OCI</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>Registros de imágenes: Docker Hub, GHCR, ECR, ACR, GAR y Harbor como registro privado</t>
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Application Bundles e Infraestructura Declarativa</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Helm: charts, templates, values, hooks. El catálogo de Helm (Artifact Hub) como ecosistema de distribución</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>Contenedores y Ecosistema OCI</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>Seguridad de imágenes: CVE scanning con Trivy/Grype, image signing con Cosign y generación de SBOM</t>
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Application Bundles e Infraestructura Declarativa</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Helm + Kustomize: helm-secrets, helm-diff. Combinar render de Helm con overlays Kustomize por entorno</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B64" s="5" t="inlineStr">
-        <is>
-          <t>Contenedores y Ecosistema OCI</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>Builds in-cluster: kaniko, buildah y Paketo Buildpacks para entornos sin Docker daemon</t>
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Application Bundles e Infraestructura Declarativa</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Caso real: charts que despliegan operators (kube-prometheus-stack, Grafana Operator). Se profundiza en la Sesión 24</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B65" s="5" t="inlineStr">
-        <is>
-          <t>Contenedores y Ecosistema OCI</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>Optimización: reducción de tamaño, gestión de capas, secrets en build time y multi-platform builds</t>
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Application Bundles e Infraestructura Declarativa</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>ExternalDNS: providers (Route53, CloudDNS, Cloudflare), anotaciones y políticas de sync</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B66" s="5" t="inlineStr">
-        <is>
-          <t>Contenedores y Ecosistema OCI</t>
-        </is>
-      </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>OCI Artifacts: almacenamiento de Helm charts, políticas OPA y otros artefactos en registros OCI</t>
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Application Bundles e Infraestructura Declarativa</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>cert-manager: Issuers, ClusterIssuers, Let's Encrypt, ACME DNS-01/HTTP-01, renovación automática</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B67" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C67" s="5" t="inlineStr">
-        <is>
-          <t>Introducción · Control Plane: kube-apiserver, etcd, kube-scheduler, controller-manager, cloud-controller-manager</t>
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Application Bundles e Infraestructura Declarativa</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Crossplane: Providers, Managed Resources, Compositions, XRDs. Comparativa con Terraform</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B68" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C68" s="5" t="inlineStr">
-        <is>
-          <t>Introducción · Data Plane: kubelet, kube-proxy, container runtime y comunicación entre nodos</t>
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Application Bundles e Infraestructura Declarativa</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Crossplane avanzado: Composition Functions, EnvironmentConfigs, integración con ArgoCD</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B69" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C69" s="5" t="inlineStr">
-        <is>
-          <t>Clusters locales · kind (Kubernetes in Docker): configuración multi-nodo, networking y uso en CI</t>
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Secretos: Vault y External Secrets</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Vault · Arquitectura: server, agents, backends de almacenamiento y alta disponibilidad</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B70" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>Building Blocks · Pods: ciclo de vida, init containers, sidecar pattern y ephemeral containers</t>
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Secretos: Vault y External Secrets</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Vault · Auth methods en Kubernetes: Kubernetes Auth, JWT/OIDC, AppRole y cloud IAM</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B71" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C71" s="5" t="inlineStr">
-        <is>
-          <t>Building Blocks · Workloads: Deployment, StatefulSet, DaemonSet, Job, CronJob y ReplicaSet</t>
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Secretos: Vault y External Secrets</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Vault · Secrets Engines: KV v1/v2, Dynamic Secrets (database, AWS, Azure), PKI y Transit</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>Building Blocks · Configuración: ConfigMap, Secret (tipos, encriptación at rest), env vars y volúmenes</t>
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Secretos: Vault y External Secrets</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Vault · Vault Agent: auto-auth, template rendering, sidecar injection. Vault Secrets Operator (VSO)</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>Building Blocks · Namespace, Labels, Selectors, Annotations, Finalizers y OwnerReferences</t>
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Secretos: Vault y External Secrets</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Vault · Políticas (HCL), namespaces, auditing, DR con Raft y auto-unseal con KMS (AWS, Azure, GCP)</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B74" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C74" s="5" t="inlineStr">
-        <is>
-          <t>Building Blocks · Scheduling: node/pod affinity, taints, tolerations, topology spread y priority classes</t>
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Secretos: Vault y External Secrets</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>External Secrets · ExternalSecret, SecretStore, ClusterSecretStore y refresh intervals</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B75" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C75" s="5" t="inlineStr">
-        <is>
-          <t>Building Blocks · Resource management: requests, limits, LimitRange, ResourceQuota y QoS classes</t>
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Secretos: Vault y External Secrets</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>External Secrets · Providers: AWS Secrets Manager, Azure Key Vault, GCP Secret Manager y Vault</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B76" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C76" s="5" t="inlineStr">
-        <is>
-          <t>Almacenamiento · PersistentVolume, PersistentVolumeClaim, StorageClass, dynamic provisioning y CSI (EBS, Azure Disk, GCE PD)</t>
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Secretos: Vault y External Secrets</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>External Secrets · Patrones avanzados: secret templating, generators, pushSecret e integración con GitOps</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="8" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="B77" s="5" t="inlineStr">
-        <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
-        </is>
-      </c>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>Networking · Services (ClusterIP, NodePort, LoadBalancer, Headless), Ingress, Gateway API, CNI (Calico, Cilium) y NetworkPolicy</t>
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Secretos: Vault y External Secrets</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Secret Management · Sealed Secrets, SOPS y comparativa de patrones por madurez</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+          <t>Observabilidad (I): Métricas</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Networking · DNS interno: CoreDNS, resolución de servicios y customización de zonas</t>
+          <t>Los tres pilares: métricas, logs, trazas. Correlación entre señales</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+          <t>Observabilidad (I): Métricas</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Autenticación · RBAC: ServiceAccounts, Roles, ClusterRoles, Bindings y principio de mínimo privilegio</t>
+          <t>Prometheus: arquitectura, scraping, PromQL, service discovery, Alertmanager</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+          <t>Observabilidad (I): Métricas</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Autenticación · certificados X.509, OIDC, webhook auth, bound SA tokens y admission controllers (Gatekeeper, Kyverno, PSA)</t>
+          <t>Prometheus Operator: ServiceMonitor, PodMonitor, recording rules, alerting rules. Thanos para HA</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>Kubernetes Core: Arquitectura y Building Blocks</t>
+          <t>Observabilidad (II): Grafana y Logs</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Cluster desde cero · etcd, kube-apiserver, scheduler, controller-manager, kubelet, kube-proxy: configuración manual, PKI y TLS bootstrapping</t>
+          <t>Grafana: datasources, dashboards, variables, alerting. Grafana as Code (grafonnet, Terraform)</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B82" s="3" t="inlineStr">
-        <is>
-          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
-        </is>
-      </c>
-      <c r="C82" s="3" t="inlineStr">
-        <is>
-          <t>EKS (AWS): arquitectura, node groups (managed, self-managed, Fargate), eksctl</t>
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Observabilidad (II): Grafana y Logs</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Loki: arquitectura, LogQL (mismo modelo mental que PromQL), labels vs indexación de texto completo</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B83" s="3" t="inlineStr">
-        <is>
-          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
-        </is>
-      </c>
-      <c r="C83" s="3" t="inlineStr">
-        <is>
-          <t>EKS Add-ons: AWS Load Balancer Controller, EBS/EFS CSI, VPC CNI, ExternalDNS</t>
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Observabilidad (II): Grafana y Logs</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>Promtail: recolección de logs de los Pods y envío a Loki</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B84" s="3" t="inlineStr">
-        <is>
-          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
-        </is>
-      </c>
-      <c r="C84" s="3" t="inlineStr">
-        <is>
-          <t>EKS Seguridad: IRSA, EKS Pod Identity, KMS encryption y audit logging</t>
+      <c r="A84" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Observabilidad (II): Grafana y Logs</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Grafana Explore: consulta y filtrado de logs por label en tiempo real</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B85" s="3" t="inlineStr">
-        <is>
-          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
-        </is>
-      </c>
-      <c r="C85" s="3" t="inlineStr">
-        <is>
-          <t>GKE: Standard vs Autopilot, node pools, Workload Identity y VPC-native networking</t>
+      <c r="A85" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>OpenTelemetry: especificación OTLP, SDK, auto-instrumentación de la app sin tocar código</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B86" s="3" t="inlineStr">
-        <is>
-          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
-        </is>
-      </c>
-      <c r="C86" s="3" t="inlineStr">
-        <is>
-          <t>GKE Add-ons: Cloud Operations, Config Connector, GKE Gateway y Fleet Management</t>
+      <c r="A86" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>OpenTelemetry Collector: pipeline de receivers, processors y exporters</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B87" s="3" t="inlineStr">
-        <is>
-          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
-        </is>
-      </c>
-      <c r="C87" s="3" t="inlineStr">
-        <is>
-          <t>AKS: arquitectura, AAD/Entra ID integration, Managed Identities y Azure CNI</t>
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Tempo: backend de trazas distribuidas, trace ID, spans, integración con Grafana</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B88" s="3" t="inlineStr">
-        <is>
-          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
-        </is>
-      </c>
-      <c r="C88" s="3" t="inlineStr">
-        <is>
-          <t>AKS Add-ons: Azure Monitor, CSI drivers (Disk/Files/Blob), AGIC y Azure Policy</t>
+      <c r="A88" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Mimir: métricas a escala/federadas (mención breve, complementa Prometheus de la Sesión 19)</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B89" s="3" t="inlineStr">
-        <is>
-          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
-        </is>
-      </c>
-      <c r="C89" s="3" t="inlineStr">
-        <is>
-          <t>AKS Seguridad: Workload Identity, Azure Key Vault CSI Provider y Defender for Containers</t>
+      <c r="A89" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Correlación end-to-end: exemplars, salto métrica→traza→logs en un mismo dashboard</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B90" s="3" t="inlineStr">
-        <is>
-          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
-        </is>
-      </c>
-      <c r="C90" s="3" t="inlineStr">
-        <is>
-          <t>Otros entornos: OVHcloud, DigitalOcean DOKS, Linode LKE, on-premises (k3s, k0s, Rancher, OpenShift)</t>
+      <c r="A90" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Git y GitOps con ArgoCD</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Git para el repositorio de manifiestos: ramas, commits, PR, revisión y conflictos sencillos; sin Git avanzado</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B91" s="3" t="inlineStr">
-        <is>
-          <t>Kubernetes en Producción: clústeres gestionados multi-cloud</t>
-        </is>
-      </c>
-      <c r="C91" s="3" t="inlineStr">
-        <is>
-          <t>Aprovisionamiento IaC: Terraform modules para EKS, GKE y AKS. Comparativa multi-cloud</t>
+      <c r="A91" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Git y GitOps con ArgoCD</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Principios GitOps: declarativo, versionado, automatizado, reconciliado. Pull vs Push model</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B92" s="3" t="inlineStr">
-        <is>
-          <t>Application Bundles e Infraestructura Declarativa</t>
-        </is>
-      </c>
-      <c r="C92" s="3" t="inlineStr">
-        <is>
-          <t>Kustomize: bases, overlays, patches, generators y transformers. 2 ejemplos prácticos (dev/prod)</t>
+      <c r="A92" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Git y GitOps con ArgoCD</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>ArgoCD: Applications, AppProjects, ApplicationSets, sync policies, waves, hooks y RBAC</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B93" s="3" t="inlineStr">
-        <is>
-          <t>Application Bundles e Infraestructura Declarativa</t>
-        </is>
-      </c>
-      <c r="C93" s="3" t="inlineStr">
-        <is>
-          <t>Helm: charts, templates, values, hooks. El catálogo de Helm (Artifact Hub) como ecosistema de distribución</t>
+      <c r="A93" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Git y GitOps con ArgoCD</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>ArgoCD avanzado: multi-tenancy, SSO, App of Apps, ApplicationSet generators y notifications</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B94" s="3" t="inlineStr">
-        <is>
-          <t>Application Bundles e Infraestructura Declarativa</t>
-        </is>
-      </c>
-      <c r="C94" s="3" t="inlineStr">
-        <is>
-          <t>Helm + Kustomize: helm-secrets, helm-diff. Combinar render de Helm con overlays Kustomize por entorno</t>
+      <c r="A94" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Git y GitOps con ArgoCD</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Práctica: modificar un manifiesto, revisar el PR, sincronizar con ArgoCD y observar la reconciliación</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B95" s="3" t="inlineStr">
-        <is>
-          <t>Application Bundles e Infraestructura Declarativa</t>
-        </is>
-      </c>
-      <c r="C95" s="3" t="inlineStr">
-        <is>
-          <t>Caso real: charts que despliegan operators (kube-prometheus-stack, Grafana Operator). Se profundiza en la Sesión 24</t>
+      <c r="A95" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines CI/CD: Prow y Tekton</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>Git aplicado a CI: cambios y PR como disparadores de validaciones y pipelines</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B96" s="3" t="inlineStr">
-        <is>
-          <t>Application Bundles e Infraestructura Declarativa</t>
-        </is>
-      </c>
-      <c r="C96" s="3" t="inlineStr">
-        <is>
-          <t>ExternalDNS: providers (Route53, CloudDNS, Cloudflare), anotaciones y políticas de sync</t>
+      <c r="A96" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines CI/CD: Prow y Tekton</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>Prow: arquitectura CI nativa en Kubernetes, plugins, Tide, Deck dashboard y ProwJobs</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B97" s="3" t="inlineStr">
-        <is>
-          <t>Application Bundles e Infraestructura Declarativa</t>
-        </is>
-      </c>
-      <c r="C97" s="3" t="inlineStr">
-        <is>
-          <t>cert-manager: Issuers, ClusterIssuers, Let's Encrypt, ACME DNS-01/HTTP-01, renovación automática</t>
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines CI/CD: Prow y Tekton</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>Tekton: Tasks, Pipelines, PipelineRuns, Workspaces, Triggers y Tekton Chains</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B98" s="3" t="inlineStr">
-        <is>
-          <t>Application Bundles e Infraestructura Declarativa</t>
-        </is>
-      </c>
-      <c r="C98" s="3" t="inlineStr">
-        <is>
-          <t>Crossplane: Providers, Managed Resources, Compositions, XRDs. Comparativa con Terraform</t>
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>Pipelines CI/CD: Prow y Tekton</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>Integración Tekton + ArgoCD para workflows CI/CD end-to-end en Kubernetes</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B99" s="3" t="inlineStr">
-        <is>
-          <t>Application Bundles e Infraestructura Declarativa</t>
-        </is>
-      </c>
-      <c r="C99" s="3" t="inlineStr">
-        <is>
-          <t>Crossplane avanzado: Composition Functions, EnvironmentConfigs, integración con ArgoCD</t>
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>Networking Avanzado (Service Mesh)</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Traefik: IngressRoute CRDs, middlewares, TLS automático, dashboard y métricas</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B100" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Secretos: Vault y External Secrets</t>
-        </is>
-      </c>
-      <c r="C100" s="3" t="inlineStr">
-        <is>
-          <t>Vault · Arquitectura: server, agents, backends de almacenamiento y alta disponibilidad</t>
+      <c r="A100" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>Networking Avanzado (Service Mesh)</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Traefik avanzado: TCP/UDP routing, rate limiting, circuit breaker, canary con TraefikService</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B101" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Secretos: Vault y External Secrets</t>
-        </is>
-      </c>
-      <c r="C101" s="3" t="inlineStr">
-        <is>
-          <t>Vault · Auth methods en Kubernetes: Kubernetes Auth, JWT/OIDC, AppRole y cloud IAM</t>
+      <c r="A101" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>Networking Avanzado (Service Mesh)</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Istio: arquitectura (Istiod + Envoy sidecars), mTLS automático y observabilidad integrada</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B102" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Secretos: Vault y External Secrets</t>
-        </is>
-      </c>
-      <c r="C102" s="3" t="inlineStr">
-        <is>
-          <t>Vault · Secrets Engines: KV v1/v2, Dynamic Secrets (database, AWS, Azure), PKI y Transit</t>
+      <c r="A102" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>Networking Avanzado (Service Mesh)</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>Istio traffic: VirtualServices, DestinationRules, Gateways, traffic shifting, fault injection</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B103" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Secretos: Vault y External Secrets</t>
-        </is>
-      </c>
-      <c r="C103" s="3" t="inlineStr">
-        <is>
-          <t>Vault · Vault Agent: auto-auth, template rendering, sidecar injection. Vault Secrets Operator (VSO)</t>
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>Networking Avanzado (Service Mesh)</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>Istio seguridad: AuthorizationPolicies, PeerAuthentication, circuit breaking, Kiali</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B104" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Secretos: Vault y External Secrets</t>
-        </is>
-      </c>
-      <c r="C104" s="3" t="inlineStr">
-        <is>
-          <t>Vault · Políticas (HCL), namespaces, auditing, DR con Raft y auto-unseal con KMS (AWS, Azure, GCP)</t>
+      <c r="A104" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>Networking Avanzado (Service Mesh)</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>Ambient Mesh (Istio): modo sin sidecar, ztunnel, waypoints y migración</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B105" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Secretos: Vault y External Secrets</t>
-        </is>
-      </c>
-      <c r="C105" s="3" t="inlineStr">
-        <is>
-          <t>External Secrets · ExternalSecret, SecretStore, ClusterSecretStore y refresh intervals</t>
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>Entrega Progresiva y Escalado</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Estrategias: rolling update, blue/green, canary, A/B testing y trade-offs</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B106" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Secretos: Vault y External Secrets</t>
-        </is>
-      </c>
-      <c r="C106" s="3" t="inlineStr">
-        <is>
-          <t>External Secrets · Providers: AWS Secrets Manager, Azure Key Vault, GCP Secret Manager y Vault</t>
+      <c r="A106" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>Entrega Progresiva y Escalado</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>Argo Rollouts: canary con análisis automatizado, blue-green, integración Istio/Traefik + Prometheus</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B107" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Secretos: Vault y External Secrets</t>
-        </is>
-      </c>
-      <c r="C107" s="3" t="inlineStr">
-        <is>
-          <t>External Secrets · Patrones avanzados: secret templating, generators, pushSecret e integración con GitOps</t>
+      <c r="A107" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>Entrega Progresiva y Escalado</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Progressive delivery: Feature flags (Flagger/OpenFeature), métricas como gates, rollback automático</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="6" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="B108" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Secretos: Vault y External Secrets</t>
-        </is>
-      </c>
-      <c r="C108" s="3" t="inlineStr">
-        <is>
-          <t>Secret Management · Sealed Secrets, SOPS y comparativa de patrones por madurez</t>
+      <c r="A108" s="8" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>Entrega Progresiva y Escalado</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>HPA: métricas CPU/memory, custom metrics (Prometheus Adapter), scaling behavior</t>
         </is>
       </c>
     </row>
@@ -4246,12 +4246,12 @@
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>Observabilidad (I): Métricas</t>
+          <t>Entrega Progresiva y Escalado</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Los tres pilares: métricas, logs, trazas. Correlación entre señales</t>
+          <t>VPA: modos (Off/Initial/Auto), recomendaciones y limitaciones</t>
         </is>
       </c>
     </row>
@@ -4263,12 +4263,12 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>Observabilidad (I): Métricas</t>
+          <t>Entrega Progresiva y Escalado</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>Prometheus: arquitectura, scraping, PromQL, service discovery, Alertmanager</t>
+          <t>KEDA: ScaledObject, ScaledJob, triggers (Kafka, SQS, Prometheus, cron) y cooldown</t>
         </is>
       </c>
     </row>
@@ -4280,996 +4280,503 @@
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>Observabilidad (I): Métricas</t>
+          <t>Entrega Progresiva y Escalado</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Prometheus Operator: ServiceMonitor, PodMonitor, recording rules, alerting rules. Thanos para HA</t>
+          <t>Cluster Autoscaler vs Karpenter: node pools, scale-from-zero, cost optimization</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B112" s="5" t="inlineStr">
-        <is>
-          <t>Observabilidad (II): Grafana y Logs</t>
-        </is>
-      </c>
-      <c r="C112" s="5" t="inlineStr">
-        <is>
-          <t>Grafana: datasources, dashboards, variables, alerting. Grafana as Code (grafonnet, Terraform)</t>
+      <c r="A112" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>Go: de cero a controlador de Kubernetes</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>Fundamentos de Go: tipos, structs, interfaces, goroutines, channels, manejo de errores idiomático</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B113" s="5" t="inlineStr">
-        <is>
-          <t>Observabilidad (II): Grafana y Logs</t>
-        </is>
-      </c>
-      <c r="C113" s="5" t="inlineStr">
-        <is>
-          <t>Loki: arquitectura, LogQL (mismo modelo mental que PromQL), labels vs indexación de texto completo</t>
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>Go: de cero a controlador de Kubernetes</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>client-go: clientset, kubeconfig, serialización, listar/filtrar/crear recursos de la API</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B114" s="5" t="inlineStr">
-        <is>
-          <t>Observabilidad (II): Grafana y Logs</t>
-        </is>
-      </c>
-      <c r="C114" s="5" t="inlineStr">
-        <is>
-          <t>Promtail: recolección de logs de los Pods y envío a Loki</t>
+      <c r="A114" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>Go: de cero a controlador de Kubernetes</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>controller-runtime: reconciliation loop, informers, predicates (fundamentos, sin construir el operator todavía)</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B115" s="5" t="inlineStr">
-        <is>
-          <t>Observabilidad (II): Grafana y Logs</t>
-        </is>
-      </c>
-      <c r="C115" s="5" t="inlineStr">
-        <is>
-          <t>Grafana Explore: consulta y filtrado de logs por label en tiempo real</t>
+      <c r="A115" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>Go: de cero a controlador de Kubernetes</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>CLIs y tooling: cobra/viper, logging estructurado, go test, mocks con testify, golangci-lint</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B116" s="5" t="inlineStr">
-        <is>
-          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
-        </is>
-      </c>
-      <c r="C116" s="5" t="inlineStr">
-        <is>
-          <t>OpenTelemetry: especificación OTLP, SDK, auto-instrumentación de la app sin tocar código</t>
+      <c r="A116" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>Construcción de Operators</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>Operator SDK (Go): scaffolding, CRD design, controller implementation y webhooks</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B117" s="5" t="inlineStr">
-        <is>
-          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
-        </is>
-      </c>
-      <c r="C117" s="5" t="inlineStr">
-        <is>
-          <t>OpenTelemetry Collector: pipeline de receivers, processors y exporters</t>
+      <c r="A117" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>Construcción de Operators</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>kubebuilder: reconciliation patterns, finalizers, status conditions y API versioning</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B118" s="5" t="inlineStr">
-        <is>
-          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
-        </is>
-      </c>
-      <c r="C118" s="5" t="inlineStr">
-        <is>
-          <t>Tempo: backend de trazas distribuidas, trace ID, spans, integración con Grafana</t>
+      <c r="A118" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>Construcción de Operators</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>Operadores de producción: leader election, metrics, testing (envtest) y OLM</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B119" s="5" t="inlineStr">
-        <is>
-          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
-        </is>
-      </c>
-      <c r="C119" s="5" t="inlineStr">
-        <is>
-          <t>Mimir: métricas a escala/federadas (mención breve, complementa Prometheus de la Sesión 19)</t>
+      <c r="A119" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Clústeres y Serverless</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>Cluster API (CAPI): arquitectura, providers (AWS/Azure/GCP), lifecycle y upgrades</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B120" s="5" t="inlineStr">
-        <is>
-          <t>Observabilidad (III): OpenTelemetry, Tempo y Correlación</t>
-        </is>
-      </c>
-      <c r="C120" s="5" t="inlineStr">
-        <is>
-          <t>Correlación end-to-end: exemplars, salto métrica→traza→logs en un mismo dashboard</t>
+      <c r="A120" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Clústeres y Serverless</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>Rancher Fleet y ArgoCD ApplicationSets para gestión de flotas de clusters</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B121" s="5" t="inlineStr">
-        <is>
-          <t>GitOps y Pipelines CI/CD</t>
-        </is>
-      </c>
-      <c r="C121" s="5" t="inlineStr">
-        <is>
-          <t>Principios GitOps: declarativo, versionado, automatizado, reconciliado. Pull vs Push model</t>
+      <c r="A121" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Clústeres y Serverless</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>Upgrade strategies: rolling upgrades, ventanas de mantenimiento y node drain</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B122" s="5" t="inlineStr">
-        <is>
-          <t>GitOps y Pipelines CI/CD</t>
-        </is>
-      </c>
-      <c r="C122" s="5" t="inlineStr">
-        <is>
-          <t>ArgoCD: Applications, AppProjects, ApplicationSets, sync policies, waves, hooks y RBAC</t>
+      <c r="A122" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Clústeres y Serverless</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>Knative Serving: auto-scaling a cero, revision routing y traffic splitting</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B123" s="5" t="inlineStr">
-        <is>
-          <t>GitOps y Pipelines CI/CD</t>
-        </is>
-      </c>
-      <c r="C123" s="5" t="inlineStr">
-        <is>
-          <t>ArgoCD avanzado: multi-tenancy, SSO, App of Apps, ApplicationSet generators y notifications</t>
+      <c r="A123" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Clústeres y Serverless</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>Virtual Kubelet: nodos virtuales con Fargate, ACI y Cloud Run</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B124" s="5" t="inlineStr">
-        <is>
-          <t>GitOps y Pipelines CI/CD</t>
-        </is>
-      </c>
-      <c r="C124" s="5" t="inlineStr">
-        <is>
-          <t>ArgoCD Image Updater y Argo Rollouts: patrones de Progressive Delivery con análisis automático</t>
+      <c r="A124" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>Hosted Control Planes</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>HyperShift (Red Hat): arquitectura, hosted clusters y node pools</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B125" s="5" t="inlineStr">
-        <is>
-          <t>GitOps y Pipelines CI/CD</t>
-        </is>
-      </c>
-      <c r="C125" s="5" t="inlineStr">
-        <is>
-          <t>Prow: arquitectura CI nativa en Kubernetes, plugins, Tide, Deck dashboard y ProwJobs</t>
+      <c r="A125" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>Hosted Control Planes</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>vCluster: clusters virtuales ligeros, sincronización y multi-tenancy</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B126" s="5" t="inlineStr">
-        <is>
-          <t>GitOps y Pipelines CI/CD</t>
-        </is>
-      </c>
-      <c r="C126" s="5" t="inlineStr">
-        <is>
-          <t>Tekton: Tasks, Pipelines, PipelineRuns, Workspaces, Triggers y Tekton Chains</t>
+      <c r="A126" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>Hosted Control Planes</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>Kamaji: tenant control planes, datastores y gestión de flota</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B127" s="5" t="inlineStr">
-        <is>
-          <t>GitOps y Pipelines CI/CD</t>
-        </is>
-      </c>
-      <c r="C127" s="5" t="inlineStr">
-        <is>
-          <t>Integración Tekton + ArgoCD para workflows CI/CD end-to-end en Kubernetes</t>
+      <c r="A127" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>Multi-cluster y Multi-cloud</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>Arquitecturas: hub-and-spoke, peer-to-peer, federación</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B128" s="5" t="inlineStr">
-        <is>
-          <t>Networking Avanzado (Service Mesh)</t>
-        </is>
-      </c>
-      <c r="C128" s="5" t="inlineStr">
-        <is>
-          <t>Traefik: IngressRoute CRDs, middlewares, TLS automático, dashboard y métricas</t>
+      <c r="A128" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>Multi-cluster y Multi-cloud</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>Open Cluster Management (OCM), Rancher MCM y ArgoCD multicluster</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B129" s="5" t="inlineStr">
-        <is>
-          <t>Networking Avanzado (Service Mesh)</t>
-        </is>
-      </c>
-      <c r="C129" s="5" t="inlineStr">
-        <is>
-          <t>Traefik avanzado: TCP/UDP routing, rate limiting, circuit breaker, canary con TraefikService</t>
+      <c r="A129" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>Multi-cluster y Multi-cloud</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>Istio multicluster (primary-remote, multi-primary)</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B130" s="5" t="inlineStr">
-        <is>
-          <t>Networking Avanzado (Service Mesh)</t>
-        </is>
-      </c>
-      <c r="C130" s="5" t="inlineStr">
-        <is>
-          <t>Istio: arquitectura (Istiod + Envoy sidecars), mTLS automático y observabilidad integrada</t>
+      <c r="A130" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>Multi-cluster y Multi-cloud</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>Cilium Cluster Mesh: tunneling, shared services y network policies globales</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B131" s="5" t="inlineStr">
-        <is>
-          <t>Networking Avanzado (Service Mesh)</t>
-        </is>
-      </c>
-      <c r="C131" s="5" t="inlineStr">
-        <is>
-          <t>Istio traffic: VirtualServices, DestinationRules, Gateways, traffic shifting, fault injection</t>
+      <c r="A131" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>Multi-cluster y Multi-cloud</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>Submariner: cross-cluster networking, service discovery y globalnet</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B132" s="5" t="inlineStr">
-        <is>
-          <t>Networking Avanzado (Service Mesh)</t>
-        </is>
-      </c>
-      <c r="C132" s="5" t="inlineStr">
-        <is>
-          <t>Istio seguridad: AuthorizationPolicies, PeerAuthentication, circuit breaking, Kiali</t>
+      <c r="A132" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>Multi-cluster y Multi-cloud</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>Crossplane como plano de control universal, políticas OPA y ESO multi-cloud</t>
         </is>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="8" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="B133" s="5" t="inlineStr">
-        <is>
-          <t>Networking Avanzado (Service Mesh)</t>
-        </is>
-      </c>
-      <c r="C133" s="5" t="inlineStr">
-        <is>
-          <t>Ambient Mesh (Istio): modo sin sidecar, ztunnel, waypoints y migración</t>
+      <c r="A133" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>Multi-cluster y Multi-cloud</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>Disaster Recovery: Velero, replicación de estado, RPO/RTO y failover automático</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="8" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>PF</t>
         </is>
       </c>
       <c r="B134" s="5" t="inlineStr">
         <is>
-          <t>Entrega Progresiva y Escalado</t>
+          <t>Plataforma Interna de Desarrollo end-to-end</t>
         </is>
       </c>
       <c r="C134" s="5" t="inlineStr">
         <is>
-          <t>Estrategias: rolling update, blue/green, canary, A/B testing y trade-offs</t>
+          <t>Aprovisionamiento de la infraestructura base con Terraform sobre uno o varios proveedores cloud</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="8" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>PF</t>
         </is>
       </c>
       <c r="B135" s="5" t="inlineStr">
         <is>
-          <t>Entrega Progresiva y Escalado</t>
+          <t>Plataforma Interna de Desarrollo end-to-end</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>Argo Rollouts: canary con análisis automatizado, blue-green, integración Istio/Traefik + Prometheus</t>
+          <t>Despliegue y configuración de un clúster Kubernetes gestionado</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="8" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>PF</t>
         </is>
       </c>
       <c r="B136" s="5" t="inlineStr">
         <is>
-          <t>Entrega Progresiva y Escalado</t>
+          <t>Plataforma Interna de Desarrollo end-to-end</t>
         </is>
       </c>
       <c r="C136" s="5" t="inlineStr">
         <is>
-          <t>Progressive delivery: Feature flags (Flagger/OpenFeature), métricas como gates, rollback automático</t>
+          <t>Flujo GitOps con ArgoCD para el ciclo de vida de las aplicaciones de plataforma</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="8" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>PF</t>
         </is>
       </c>
       <c r="B137" s="5" t="inlineStr">
         <is>
-          <t>Entrega Progresiva y Escalado</t>
+          <t>Plataforma Interna de Desarrollo end-to-end</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>HPA: métricas CPU/memory, custom metrics (Prometheus Adapter), scaling behavior</t>
+          <t>Gestión de secretos con Vault y/o External Secrets Operator</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="8" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>PF</t>
         </is>
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>Entrega Progresiva y Escalado</t>
+          <t>Plataforma Interna de Desarrollo end-to-end</t>
         </is>
       </c>
       <c r="C138" s="5" t="inlineStr">
         <is>
-          <t>VPA: modos (Off/Initial/Auto), recomendaciones y limitaciones</t>
+          <t>Stack de observabilidad (métricas, logs, trazas) y alerting</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="8" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>PF</t>
         </is>
       </c>
       <c r="B139" s="5" t="inlineStr">
         <is>
-          <t>Entrega Progresiva y Escalado</t>
+          <t>Plataforma Interna de Desarrollo end-to-end</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>KEDA: ScaledObject, ScaledJob, triggers (Kafka, SQS, Prometheus, cron) y cooldown</t>
+          <t>Entrega progresiva (canary o blue/green) con rollback automático basado en métricas</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="8" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>PF</t>
         </is>
       </c>
       <c r="B140" s="5" t="inlineStr">
         <is>
-          <t>Entrega Progresiva y Escalado</t>
+          <t>Plataforma Interna de Desarrollo end-to-end</t>
         </is>
       </c>
       <c r="C140" s="5" t="inlineStr">
-        <is>
-          <t>Cluster Autoscaler vs Karpenter: node pools, scale-from-zero, cost optimization</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B141" s="3" t="inlineStr">
-        <is>
-          <t>Go: de cero a controlador de Kubernetes</t>
-        </is>
-      </c>
-      <c r="C141" s="3" t="inlineStr">
-        <is>
-          <t>Fundamentos de Go: tipos, structs, interfaces, goroutines, channels, manejo de errores idiomático</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B142" s="3" t="inlineStr">
-        <is>
-          <t>Go: de cero a controlador de Kubernetes</t>
-        </is>
-      </c>
-      <c r="C142" s="3" t="inlineStr">
-        <is>
-          <t>client-go: clientset, kubeconfig, serialización, listar/filtrar/crear recursos de la API</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B143" s="3" t="inlineStr">
-        <is>
-          <t>Go: de cero a controlador de Kubernetes</t>
-        </is>
-      </c>
-      <c r="C143" s="3" t="inlineStr">
-        <is>
-          <t>controller-runtime: reconciliation loop, informers, predicates (fundamentos, sin construir el operator todavía)</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B144" s="3" t="inlineStr">
-        <is>
-          <t>Go: de cero a controlador de Kubernetes</t>
-        </is>
-      </c>
-      <c r="C144" s="3" t="inlineStr">
-        <is>
-          <t>CLIs y tooling: cobra/viper, logging estructurado, go test, mocks con testify, golangci-lint</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B145" s="3" t="inlineStr">
-        <is>
-          <t>Construcción de Operators</t>
-        </is>
-      </c>
-      <c r="C145" s="3" t="inlineStr">
-        <is>
-          <t>Operator SDK (Go): scaffolding, CRD design, controller implementation y webhooks</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B146" s="3" t="inlineStr">
-        <is>
-          <t>Construcción de Operators</t>
-        </is>
-      </c>
-      <c r="C146" s="3" t="inlineStr">
-        <is>
-          <t>kubebuilder: reconciliation patterns, finalizers, status conditions y API versioning</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B147" s="3" t="inlineStr">
-        <is>
-          <t>Construcción de Operators</t>
-        </is>
-      </c>
-      <c r="C147" s="3" t="inlineStr">
-        <is>
-          <t>Operadores de producción: leader election, metrics, testing (envtest) y OLM</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B148" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Clústeres y Serverless</t>
-        </is>
-      </c>
-      <c r="C148" s="3" t="inlineStr">
-        <is>
-          <t>Cluster API (CAPI): arquitectura, providers (AWS/Azure/GCP), lifecycle y upgrades</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B149" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Clústeres y Serverless</t>
-        </is>
-      </c>
-      <c r="C149" s="3" t="inlineStr">
-        <is>
-          <t>Rancher Fleet y ArgoCD ApplicationSets para gestión de flotas de clusters</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B150" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Clústeres y Serverless</t>
-        </is>
-      </c>
-      <c r="C150" s="3" t="inlineStr">
-        <is>
-          <t>Upgrade strategies: rolling upgrades, ventanas de mantenimiento y node drain</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B151" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Clústeres y Serverless</t>
-        </is>
-      </c>
-      <c r="C151" s="3" t="inlineStr">
-        <is>
-          <t>Knative Serving: auto-scaling a cero, revision routing y traffic splitting</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B152" s="3" t="inlineStr">
-        <is>
-          <t>Gestión de Clústeres y Serverless</t>
-        </is>
-      </c>
-      <c r="C152" s="3" t="inlineStr">
-        <is>
-          <t>Virtual Kubelet: nodos virtuales con Fargate, ACI y Cloud Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B153" s="3" t="inlineStr">
-        <is>
-          <t>Hosted Control Planes</t>
-        </is>
-      </c>
-      <c r="C153" s="3" t="inlineStr">
-        <is>
-          <t>HyperShift (Red Hat): arquitectura, hosted clusters y node pools</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B154" s="3" t="inlineStr">
-        <is>
-          <t>Hosted Control Planes</t>
-        </is>
-      </c>
-      <c r="C154" s="3" t="inlineStr">
-        <is>
-          <t>vCluster: clusters virtuales ligeros, sincronización y multi-tenancy</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B155" s="3" t="inlineStr">
-        <is>
-          <t>Hosted Control Planes</t>
-        </is>
-      </c>
-      <c r="C155" s="3" t="inlineStr">
-        <is>
-          <t>Kamaji: tenant control planes, datastores y gestión de flota</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B156" s="3" t="inlineStr">
-        <is>
-          <t>Multi-cluster y Multi-cloud</t>
-        </is>
-      </c>
-      <c r="C156" s="3" t="inlineStr">
-        <is>
-          <t>Arquitecturas: hub-and-spoke, peer-to-peer, federación</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B157" s="3" t="inlineStr">
-        <is>
-          <t>Multi-cluster y Multi-cloud</t>
-        </is>
-      </c>
-      <c r="C157" s="3" t="inlineStr">
-        <is>
-          <t>Open Cluster Management (OCM), Rancher MCM y ArgoCD multicluster</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B158" s="3" t="inlineStr">
-        <is>
-          <t>Multi-cluster y Multi-cloud</t>
-        </is>
-      </c>
-      <c r="C158" s="3" t="inlineStr">
-        <is>
-          <t>Istio multicluster (primary-remote, multi-primary)</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B159" s="3" t="inlineStr">
-        <is>
-          <t>Multi-cluster y Multi-cloud</t>
-        </is>
-      </c>
-      <c r="C159" s="3" t="inlineStr">
-        <is>
-          <t>Cilium Cluster Mesh: tunneling, shared services y network policies globales</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B160" s="3" t="inlineStr">
-        <is>
-          <t>Multi-cluster y Multi-cloud</t>
-        </is>
-      </c>
-      <c r="C160" s="3" t="inlineStr">
-        <is>
-          <t>Submariner: cross-cluster networking, service discovery y globalnet</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B161" s="3" t="inlineStr">
-        <is>
-          <t>Multi-cluster y Multi-cloud</t>
-        </is>
-      </c>
-      <c r="C161" s="3" t="inlineStr">
-        <is>
-          <t>Crossplane como plano de control universal, políticas OPA y ESO multi-cloud</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="6" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="B162" s="3" t="inlineStr">
-        <is>
-          <t>Multi-cluster y Multi-cloud</t>
-        </is>
-      </c>
-      <c r="C162" s="3" t="inlineStr">
-        <is>
-          <t>Disaster Recovery: Velero, replicación de estado, RPO/RTO y failover automático</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="8" t="inlineStr">
-        <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="B163" s="5" t="inlineStr">
-        <is>
-          <t>Plataforma Interna de Desarrollo end-to-end</t>
-        </is>
-      </c>
-      <c r="C163" s="5" t="inlineStr">
-        <is>
-          <t>Aprovisionamiento de la infraestructura base con Terraform sobre uno o varios proveedores cloud</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="8" t="inlineStr">
-        <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="B164" s="5" t="inlineStr">
-        <is>
-          <t>Plataforma Interna de Desarrollo end-to-end</t>
-        </is>
-      </c>
-      <c r="C164" s="5" t="inlineStr">
-        <is>
-          <t>Despliegue y configuración de un clúster Kubernetes gestionado</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" s="8" t="inlineStr">
-        <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="B165" s="5" t="inlineStr">
-        <is>
-          <t>Plataforma Interna de Desarrollo end-to-end</t>
-        </is>
-      </c>
-      <c r="C165" s="5" t="inlineStr">
-        <is>
-          <t>Flujo GitOps con ArgoCD para el ciclo de vida de las aplicaciones de plataforma</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="8" t="inlineStr">
-        <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="B166" s="5" t="inlineStr">
-        <is>
-          <t>Plataforma Interna de Desarrollo end-to-end</t>
-        </is>
-      </c>
-      <c r="C166" s="5" t="inlineStr">
-        <is>
-          <t>Gestión de secretos con Vault y/o External Secrets Operator</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="8" t="inlineStr">
-        <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="B167" s="5" t="inlineStr">
-        <is>
-          <t>Plataforma Interna de Desarrollo end-to-end</t>
-        </is>
-      </c>
-      <c r="C167" s="5" t="inlineStr">
-        <is>
-          <t>Stack de observabilidad (métricas, logs, trazas) y alerting</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="8" t="inlineStr">
-        <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="B168" s="5" t="inlineStr">
-        <is>
-          <t>Plataforma Interna de Desarrollo end-to-end</t>
-        </is>
-      </c>
-      <c r="C168" s="5" t="inlineStr">
-        <is>
-          <t>Entrega progresiva (canary o blue/green) con rollback automático basado en métricas</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="8" t="inlineStr">
-        <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="B169" s="5" t="inlineStr">
-        <is>
-          <t>Plataforma Interna de Desarrollo end-to-end</t>
-        </is>
-      </c>
-      <c r="C169" s="5" t="inlineStr">
         <is>
           <t>Documentación, golden paths y defensa del proyecto</t>
         </is>

</xml_diff>